<commit_message>
docs: ADR 019 service fee, finmodel and spec at 5%
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G6Artzpr7bcnkUftwxLCYd
</commit_message>
<xml_diff>
--- a/docs/business/finmodel.xlsx
+++ b/docs/business/finmodel.xlsx
@@ -208,7 +208,7 @@
     <t xml:space="preserve">от цены</t>
   </si>
   <si>
-    <t xml:space="preserve">Бизнес-решение 2026-10-02: 7%, ниже рыночных ~10%.</t>
+    <t xml:space="preserve">Бизнес-решение 2026-10-02: 5% (сначала 7%, снижено владельцем продукта). Рынок ~10%. В продукте — SERVICE_FEE_BPS, ADR 019.</t>
   </si>
   <si>
     <t xml:space="preserve">Комиссия с организатора</t>
@@ -265,7 +265,7 @@
     <t xml:space="preserve">от платных</t>
   </si>
   <si>
-    <t xml:space="preserve">Сбор возвращается покупателю, эквайринг не возвращается. Допущение.</t>
+    <t xml:space="preserve">Допущение. С запасом: в продукте сбор возвращается только при отмене события, при возврате по желанию покупателя он остаётся (ADR 019); эквайринг не возвращается.</t>
   </si>
   <si>
     <t xml:space="preserve">Юр. сопровождение запуска (разово, 1-й месяц)</t>
@@ -541,7 +541,7 @@
     <t xml:space="preserve">Кто платит</t>
   </si>
   <si>
-    <t xml:space="preserve">Сервисный сбор 7% (выбрано)</t>
+    <t xml:space="preserve">Сервисный сбор 5% (выбрано)</t>
   </si>
   <si>
     <t xml:space="preserve">покупатель</t>
@@ -598,7 +598,7 @@
     <t xml:space="preserve">Оборот в год, ₸</t>
   </si>
   <si>
-    <t xml:space="preserve">Наш сбор 7%, ₸</t>
+    <t xml:space="preserve">Наш сбор, ₸</t>
   </si>
   <si>
     <t xml:space="preserve">Стендап и камеди-клубы</t>
@@ -676,10 +676,10 @@
     <t xml:space="preserve">Налог 4% считается только с нашего сбора при агентской схеме (договор с организатором, мы — агент). Без неё налоговой базой может считаться весь оборот билетов — модель тогда неверна.</t>
   </si>
   <si>
-    <t xml:space="preserve">Сервисный сбор в продукте</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сейчас в продукте сумма заказа — только цена билетов. Сбор 7% нужно добавить: строка в заказе, возврат вместе с билетом, отражение в отчёте организатора. Отдельная задача.</t>
+    <t xml:space="preserve">Ставка сбора</t>
+  </si>
+  <si>
+    <t xml:space="preserve">При 5% базовый сценарий за три года не окупается: маржа с билета около 120 ₸, а эквайринг берётся со всей суммы оплаты и от ставки не зависит. Окупаемость за три года даёт ставка около 7%. Ставка — настройка продукта (SERVICE_FEE_BPS), её можно менять без кода; старые заказы сохраняют свой сбор.</t>
   </si>
   <si>
     <t xml:space="preserve">Численности рынка</t>
@@ -1446,112 +1446,112 @@
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>-1182941.076</c:v>
+                  <c:v>-1191749.34</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1558120.34158</c:v>
+                  <c:v>-1579744.6297</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1921994.6582252</c:v>
+                  <c:v>-1962272.207018</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-2244074.09930268</c:v>
+                  <c:v>-2324585.4198162</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-2540048.22087679</c:v>
+                  <c:v>-2674272.62434954</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-2807786.02500007</c:v>
+                  <c:v>-3010303.14954373</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-3045378.27069894</c:v>
+                  <c:v>-3331753.57853314</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-3334372.70728782</c:v>
+                  <c:v>-3678065.01284086</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-3597793.03448056</c:v>
+                  <c:v>-4012007.36212128</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-3833819.49899298</c:v>
+                  <c:v>-4332700.49081416</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-4058360.72063466</c:v>
+                  <c:v>-4647838.70678547</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-4272105.81397783</c:v>
+                  <c:v>-4957755.3047985</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-5157924.2761719</c:v>
+                  <c:v>-5933511.26650429</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-6069537.90601872</c:v>
+                  <c:v>-6921743.22950688</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-6964466.33207473</c:v>
+                  <c:v>-7901905.28472931</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-7723206.88956248</c:v>
+                  <c:v>-8816199.18791112</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-8424792.58500481</c:v>
+                  <c:v>-9702849.76880112</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-9066078.23524021</c:v>
+                  <c:v>-10560335.8390229</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-9644245.95272994</c:v>
+                  <c:v>-11387294.5088653</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-10391406.6613086</c:v>
+                  <c:v>-12295987.7424973</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-11082196.5316306</c:v>
+                  <c:v>-13177416.8520631</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-11713929.7528557</c:v>
+                  <c:v>-14030282.8276096</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-12328711.6708073</c:v>
+                  <c:v>-14874950.1946233</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-12927559.3636819</c:v>
+                  <c:v>-15711910.8696161</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-14075282.3647235</c:v>
+                  <c:v>-17062183.5372108</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-15304609.2324579</c:v>
+                  <c:v>-18451924.447865</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-16518458.6401282</c:v>
+                  <c:v>-19834179.58388</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-17490626.2988117</c:v>
+                  <c:v>-21099543.7636368</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-18380938.2698904</c:v>
+                  <c:v>-22325317.9055053</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-19186477.0315056</c:v>
+                  <c:v>-23510090.930985</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-19904628.6664172</c:v>
+                  <c:v>-24652598.6019318</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-20923730.532766</c:v>
+                  <c:v>-25940662.8177411</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-21861703.9844299</c:v>
+                  <c:v>-27189488.7459594</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-22716057.6206122</c:v>
+                  <c:v>-28397871.4043207</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-23554686.9586235</c:v>
+                  <c:v>-29598648.9031803</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-24378535.4563542</c:v>
+                  <c:v>-30792277.5521084</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1806,112 +1806,112 @@
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>-1279849.83552</c:v>
+                  <c:v>-1311025.9968</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1726992.1568512</c:v>
+                  <c:v>-1803880.364608</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-2126150.4503625</c:v>
+                  <c:v>-2270075.78346464</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-2348373.02860131</c:v>
+                  <c:v>-2637969.32114479</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-2457586.37088118</c:v>
+                  <c:v>-2943077.22807779</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-2443141.56984549</c:v>
+                  <c:v>-3179483.18813708</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-2295182.36882731</c:v>
+                  <c:v>-3341711.26578175</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-2364846.95082585</c:v>
+                  <c:v>-3624846.68667447</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-2319867.65107054</c:v>
+                  <c:v>-3844288.30089608</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-2150840.79961907</c:v>
+                  <c:v>-3994811.62087568</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-1926482.45088292</c:v>
+                  <c:v>-4114593.88745619</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1649282.52223989</c:v>
+                  <c:v>-4205018.44804059</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-2110384.83595662</c:v>
+                  <c:v>-4998946.14032706</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-2696299.16255622</c:v>
+                  <c:v>-5862216.84592725</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-3222609.63885885</c:v>
+                  <c:v>-6692372.86577543</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3198257.63764052</c:v>
+                  <c:v>-7216592.02403379</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-2950810.06676067</c:v>
+                  <c:v>-7616863.82578419</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-2467039.2771713</c:v>
+                  <c:v>-7885839.25851687</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-1734702.2189753</c:v>
+                  <c:v>-8016716.3329649</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-1686288.7301278</c:v>
+                  <c:v>-8527567.41856359</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-1412749.17964727</c:v>
+                  <c:v>-8913343.04765368</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-902402.7028596</c:v>
+                  <c:v>-9167553.56963261</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-323325.641527373</c:v>
+                  <c:v>-9383578.77812249</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>321389.128044906</c:v>
+                  <c:v>-9563137.01223032</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>112074.929118125</c:v>
+                  <c:v>-10474940.1622887</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-422996.078023181</c:v>
+                  <c:v>-11567727.162918</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-891776.102003129</c:v>
+                  <c:v>-12623684.242919</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-374229.660437878</c:v>
+                  <c:v>-13131658.4192539</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>484912.987466418</c:v>
+                  <c:v>-13449848.6978938</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1700363.53996308</c:v>
+                  <c:v>-13570081.558804</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>3285738.63105357</c:v>
+                  <c:v>-13484791.877354</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>3643104.32478368</c:v>
+                  <c:v>-14081759.2160711</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>4344324.52374497</c:v>
+                  <c:v>-14487687.9922053</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>5402390.60348722</c:v>
+                  <c:v>-14695360.4619922</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>6536898.35604107</c:v>
+                  <c:v>-14860563.4946386</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>7744407.90613</c:v>
+                  <c:v>-14985208.2148159</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2166,112 +2166,112 @@
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>-1134910.22</c:v>
+                  <c:v>-1238807.3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1344234.156725</c:v>
+                  <c:v>-1601249.558375</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1368414.42066462</c:v>
+                  <c:v>-1851111.81270688</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-710942.120167522</c:v>
+                  <c:v>-1686482.73009064</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>388363.174310154</c:v>
+                  <c:v>-1253188.99639351</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1974902.87249665</c:v>
+                  <c:v>-523623.452192344</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4091518.80780912</c:v>
+                  <c:v>528264.66464129</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5369860.5124716</c:v>
+                  <c:v>1070424.76940711</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7107261.22809581</c:v>
+                  <c:v>1891724.1206435</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9344836.44262621</c:v>
+                  <c:v>3017163.74446919</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11814458.749648</c:v>
+                  <c:v>4283703.85646098</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>14508006.5009241</c:v>
+                  <c:v>5686405.93953305</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>16214769.0129092</c:v>
+                  <c:v>6230400.2676647</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>17420071.1169585</c:v>
+                  <c:v>6469472.40264997</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>18857195.383366</c:v>
+                  <c:v>6849508.25291076</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>22465249.8051714</c:v>
+                  <c:v>8549617.97874687</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>26955887.0899179</c:v>
+                  <c:v>10786398.3927219</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>32385955.2671328</c:v>
+                  <c:v>13594416.981252</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>38809097.4687295</c:v>
+                  <c:v>17006292.4340111</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>42535845.5626008</c:v>
+                  <c:v>18778576.0228804</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>47166745.5660098</c:v>
+                  <c:v>21100645.7540466</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>52753279.0185539</c:v>
+                  <c:v>24003805.9213526</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>58630363.360259</c:v>
+                  <c:v>27083640.8828029</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>64787829.3100044</c:v>
+                  <c:v>30333967.0206024</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>69257310.5392079</c:v>
+                  <c:v>32330562.7389836</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>72421195.7158439</c:v>
+                  <c:v>33533266.8451621</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>75847343.0482976</c:v>
+                  <c:v>34895444.2626242</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>83206060.2363274</c:v>
+                  <c:v>38648892.8673759</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>91932395.115921</c:v>
+                  <c:v>43233946.4788198</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>102090660.290439</c:v>
+                  <c:v>48689711.5543216</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>113741542.638466</c:v>
+                  <c:v>55053089.8628358</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>120496248.748832</c:v>
+                  <c:v>58439258.459892</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>128642973.775399</c:v>
+                  <c:v>62671869.675571</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>138239959.171107</c:v>
+                  <c:v>67786338.292938</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>148165646.972965</c:v>
+                  <c:v>73100680.4336972</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>158408532.596758</c:v>
+                  <c:v>78607900.5245298</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2286,11 +2286,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="7409653"/>
-        <c:axId val="55424785"/>
+        <c:axId val="47611281"/>
+        <c:axId val="67006473"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="7409653"/>
+        <c:axId val="47611281"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2356,7 +2356,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55424785"/>
+        <c:crossAx val="67006473"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2364,7 +2364,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55424785"/>
+        <c:axId val="67006473"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2440,7 +2440,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7409653"/>
+        <c:crossAx val="47611281"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2921,39 +2921,39 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">SUM(План!$C$17:$N$17)</f>
-        <v>2568726.573975</v>
+        <v>1834804.69569643</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">SUM(План!$O$17:$Z$17)</f>
-        <v>7862605.76176415</v>
+        <v>5616146.97268868</v>
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">SUM(План!$AA$17:$AL$17)</f>
-        <v>13597198.2481116</v>
+        <v>9712284.46293688</v>
       </c>
       <c r="E8" s="8" t="n">
         <f aca="false">SUM(План!$C$41:$N$41)</f>
-        <v>9522304.06946156</v>
+        <v>6801645.76390111</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">SUM(План!$O$41:$Z$41)</f>
-        <v>27306017.0962917</v>
+        <v>19504297.9259227</v>
       </c>
       <c r="G8" s="8" t="n">
         <f aca="false">SUM(План!$AA$41:$AL$41)</f>
-        <v>47858955.7554621</v>
+        <v>34184968.3967586</v>
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">SUM(План!$C$65:$N$65)</f>
-        <v>32688642.1151743</v>
+        <v>23349030.0822673</v>
       </c>
       <c r="I8" s="8" t="n">
         <f aca="false">SUM(План!$O$65:$Z$65)</f>
-        <v>94980930.5463841</v>
+        <v>67843521.8188458</v>
       </c>
       <c r="J8" s="8" t="n">
         <f aca="false">SUM(План!$AA$65:$AL$65)</f>
-        <v>168033489.863235</v>
+        <v>120023921.330882</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2962,39 +2962,39 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">SUM(План!$C$21:$N$21)</f>
-        <v>1327894.18602217</v>
+        <v>642244.695201505</v>
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">SUM(План!$O$21:$Z$21)</f>
-        <v>4064546.45029597</v>
+        <v>1965844.43518237</v>
       </c>
       <c r="D9" s="8" t="n">
         <f aca="false">SUM(План!$AA$21:$AL$21)</f>
-        <v>7029023.90732769</v>
+        <v>3399633.31750773</v>
       </c>
       <c r="E9" s="8" t="n">
         <f aca="false">SUM(План!$C$45:$N$45)</f>
-        <v>5750717.47776011</v>
+        <v>3194981.55195941</v>
       </c>
       <c r="F9" s="8" t="n">
         <f aca="false">SUM(План!$O$45:$Z$45)</f>
-        <v>16490671.6502848</v>
+        <v>9161881.43581027</v>
       </c>
       <c r="G9" s="8" t="n">
         <f aca="false">SUM(План!$AA$45:$AL$45)</f>
-        <v>28903018.7780851</v>
+        <v>16057928.7974144</v>
       </c>
       <c r="H9" s="8" t="n">
         <f aca="false">SUM(План!$C$69:$N$69)</f>
-        <v>22508006.5009241</v>
+        <v>13686405.9395331</v>
       </c>
       <c r="I9" s="8" t="n">
         <f aca="false">SUM(План!$O$69:$Z$69)</f>
-        <v>65399822.8090803</v>
+        <v>39767561.0810694</v>
       </c>
       <c r="J9" s="8" t="n">
         <f aca="false">SUM(План!$AA$69:$AL$69)</f>
-        <v>115700703.286754</v>
+        <v>70353933.5039274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3044,39 +3044,39 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">SUM(План!$C$27:$N$27)</f>
-        <v>-4272105.81397783</v>
+        <v>-4957755.3047985</v>
       </c>
       <c r="C11" s="8" t="n">
         <f aca="false">SUM(План!$O$27:$Z$27)</f>
-        <v>-8655453.54970403</v>
+        <v>-10754155.5648176</v>
       </c>
       <c r="D11" s="8" t="n">
         <f aca="false">SUM(План!$AA$27:$AL$27)</f>
-        <v>-11450976.0926723</v>
+        <v>-15080366.6824923</v>
       </c>
       <c r="E11" s="8" t="n">
         <f aca="false">SUM(План!$C$51:$N$51)</f>
-        <v>-1649282.52223989</v>
+        <v>-4205018.44804059</v>
       </c>
       <c r="F11" s="8" t="n">
         <f aca="false">SUM(План!$O$51:$Z$51)</f>
-        <v>1970671.65028479</v>
+        <v>-5358118.56418973</v>
       </c>
       <c r="G11" s="8" t="n">
         <f aca="false">SUM(План!$AA$51:$AL$51)</f>
-        <v>7423018.7780851</v>
+        <v>-5422071.2025856</v>
       </c>
       <c r="H11" s="8" t="n">
         <f aca="false">SUM(План!$C$75:$N$75)</f>
-        <v>14508006.5009241</v>
+        <v>5686405.93953305</v>
       </c>
       <c r="I11" s="8" t="n">
         <f aca="false">SUM(План!$O$75:$Z$75)</f>
-        <v>50279822.8090803</v>
+        <v>24647561.0810694</v>
       </c>
       <c r="J11" s="8" t="n">
         <f aca="false">SUM(План!$AA$75:$AL$75)</f>
-        <v>93620703.2867539</v>
+        <v>48273933.5039274</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3085,39 +3085,39 @@
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">План!N28</f>
-        <v>-4272105.81397783</v>
+        <v>-4957755.3047985</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">План!Z28</f>
-        <v>-12927559.3636819</v>
+        <v>-15711910.8696161</v>
       </c>
       <c r="D12" s="8" t="n">
         <f aca="false">План!AL28</f>
-        <v>-24378535.4563542</v>
+        <v>-30792277.5521084</v>
       </c>
       <c r="E12" s="8" t="n">
         <f aca="false">План!N52</f>
-        <v>-1649282.52223989</v>
+        <v>-4205018.44804059</v>
       </c>
       <c r="F12" s="8" t="n">
         <f aca="false">План!Z52</f>
-        <v>321389.128044906</v>
+        <v>-9563137.01223032</v>
       </c>
       <c r="G12" s="8" t="n">
         <f aca="false">План!AL52</f>
-        <v>7744407.90613</v>
+        <v>-14985208.2148159</v>
       </c>
       <c r="H12" s="8" t="n">
         <f aca="false">План!N76</f>
-        <v>14508006.5009241</v>
+        <v>5686405.93953305</v>
       </c>
       <c r="I12" s="8" t="n">
         <f aca="false">План!Z76</f>
-        <v>64787829.3100044</v>
+        <v>30333967.0206024</v>
       </c>
       <c r="J12" s="8" t="n">
         <f aca="false">План!AL76</f>
-        <v>158408532.596758</v>
+        <v>78607900.5245298</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3164,7 +3164,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="9" t="n">
         <f aca="false">IF(COUNT(План!$C$53:$AL$53)=0,"не достигнут",MIN(План!$C$53:$AL$53))</f>
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -3185,15 +3185,15 @@
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="9" t="str">
         <f aca="false">IF(COUNT(План!$C$54:$AL$54)=0,"за 3 года нет",MIN(План!$C$54:$AL$54))</f>
-        <v>24</v>
+        <v>за 3 года нет</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="9" t="n">
         <f aca="false">IF(COUNT(План!$C$78:$AL$78)=0,"за 3 года нет",MIN(План!$C$78:$AL$78))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -3204,19 +3204,19 @@
       </c>
       <c r="B17" s="10" t="n">
         <f aca="false">-MIN(0,MIN(План!$C$28:$AL$28))</f>
-        <v>24378535.4563542</v>
+        <v>30792277.5521084</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="10" t="n">
         <f aca="false">-MIN(0,MIN(План!$C$52:$AL$52))</f>
-        <v>3222609.63885885</v>
+        <v>14985208.2148159</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="10" t="n">
         <f aca="false">-MIN(0,MIN(План!$C$76:$AL$76))</f>
-        <v>1368414.42066462</v>
+        <v>1851111.81270688</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3227,19 +3227,19 @@
       </c>
       <c r="B18" s="10" t="n">
         <f aca="false">SUM(План!$C$17:$AL$17)</f>
-        <v>24028530.5838508</v>
+        <v>17163236.131322</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="10" t="n">
         <f aca="false">SUM(План!$C$41:$AL$41)</f>
-        <v>84687276.9212153</v>
+        <v>60490912.0865824</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="10" t="n">
         <f aca="false">SUM(План!$C$65:$AL$65)</f>
-        <v>295703062.524794</v>
+        <v>211216473.231995</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -3250,19 +3250,19 @@
       </c>
       <c r="B19" s="10" t="n">
         <f aca="false">SUM(План!$C$27:$AL$27)</f>
-        <v>-24378535.4563542</v>
+        <v>-30792277.5521084</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="10" t="n">
         <f aca="false">SUM(План!$C$51:$AL$51)</f>
-        <v>7744407.90613</v>
+        <v>-14985208.2148159</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="10" t="n">
         <f aca="false">SUM(План!$C$75:$AL$75)</f>
-        <v>158408532.596758</v>
+        <v>78607900.5245298</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -3273,19 +3273,19 @@
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">'Юнит-экономика'!C21</f>
-        <v>1.1155430625</v>
+        <v>0.5395396875</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="11" t="n">
         <f aca="false">'Юнит-экономика'!D21</f>
-        <v>4.07765873777778</v>
+        <v>2.26546417777778</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="11" t="n">
         <f aca="false">'Юнит-экономика'!E21</f>
-        <v>17.8304435357143</v>
+        <v>10.8421280357143</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -3386,15 +3386,15 @@
       </c>
       <c r="C6" s="12" t="n">
         <f aca="false">C5*(Допущения!$C$6+Допущения!$C$7)</f>
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="D6" s="12" t="n">
         <f aca="false">D5*(Допущения!$C$6+Допущения!$C$7)</f>
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">E5*(Допущения!$C$6+Допущения!$C$7)</f>
-        <v>490</v>
+        <v>350</v>
       </c>
       <c r="F6" s="3"/>
     </row>
@@ -3405,15 +3405,15 @@
       </c>
       <c r="C7" s="12" t="n">
         <f aca="false">C6*(1-Допущения!$C$12)*(1-Допущения!$C$13)</f>
-        <v>305.55</v>
+        <v>218.25</v>
       </c>
       <c r="D7" s="12" t="n">
         <f aca="false">D6*(1-Допущения!$C$12)*(1-Допущения!$C$13)</f>
-        <v>366.66</v>
+        <v>261.9</v>
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">E6*(1-Допущения!$C$12)*(1-Допущения!$C$13)</f>
-        <v>427.77</v>
+        <v>305.55</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>30</v>
@@ -3426,15 +3426,15 @@
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">C5*(1+Допущения!$C$6)*Допущения!$C$23*(1-Допущения!$C$12)</f>
-        <v>120.375</v>
+        <v>118.125</v>
       </c>
       <c r="D8" s="12" t="n">
         <f aca="false">D5*(1+Допущения!$C$6)*Допущения!$D$23*(1-Допущения!$C$12)</f>
-        <v>115.56</v>
+        <v>113.4</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">E5*(1+Допущения!$C$6)*Допущения!$E$23*(1-Допущения!$C$12)</f>
-        <v>101.115</v>
+        <v>99.225</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>32</v>
@@ -3466,15 +3466,15 @@
       </c>
       <c r="C10" s="12" t="n">
         <f aca="false">C7*Допущения!$C$8</f>
-        <v>12.222</v>
+        <v>8.73</v>
       </c>
       <c r="D10" s="12" t="n">
         <f aca="false">D7*Допущения!$C$8</f>
-        <v>14.6664</v>
+        <v>10.476</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">E7*Допущения!$C$8</f>
-        <v>17.1108</v>
+        <v>12.222</v>
       </c>
       <c r="F10" s="3"/>
     </row>
@@ -3485,15 +3485,15 @@
       </c>
       <c r="C11" s="13" t="n">
         <f aca="false">C7-C8-C9-C10</f>
-        <v>157.953</v>
+        <v>76.395</v>
       </c>
       <c r="D11" s="13" t="n">
         <f aca="false">D7-D8-D9-D10</f>
-        <v>221.4336</v>
+        <v>123.024</v>
       </c>
       <c r="E11" s="13" t="n">
         <f aca="false">E7-E8-E9-E10</f>
-        <v>294.5442</v>
+        <v>179.103</v>
       </c>
       <c r="F11" s="3"/>
     </row>
@@ -3504,15 +3504,15 @@
       </c>
       <c r="C12" s="14" t="n">
         <f aca="false">IF(C5=0,0,C11/C5)</f>
-        <v>0.0315906</v>
+        <v>0.015279</v>
       </c>
       <c r="D12" s="14" t="n">
         <f aca="false">IF(D5=0,0,D11/D5)</f>
-        <v>0.0369056</v>
+        <v>0.020504</v>
       </c>
       <c r="E12" s="14" t="n">
         <f aca="false">IF(E5=0,0,E11/E5)</f>
-        <v>0.0420777428571429</v>
+        <v>0.0255861428571429</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>37</v>
@@ -3562,15 +3562,15 @@
       </c>
       <c r="C16" s="12" t="n">
         <f aca="false">C15*C11</f>
-        <v>13386.51675</v>
+        <v>6474.47625</v>
       </c>
       <c r="D16" s="12" t="n">
         <f aca="false">D15*D11</f>
-        <v>27524.19648</v>
+        <v>15291.8832</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">E15*E11</f>
-        <v>62406.552375</v>
+        <v>37947.448125</v>
       </c>
       <c r="F16" s="3"/>
     </row>
@@ -3621,15 +3621,15 @@
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">C16*C18</f>
-        <v>223108.6125</v>
+        <v>107907.9375</v>
       </c>
       <c r="D19" s="13" t="n">
         <f aca="false">D16*D18</f>
-        <v>611648.810666667</v>
+        <v>339819.626666667</v>
       </c>
       <c r="E19" s="13" t="n">
         <f aca="false">E16*E18</f>
-        <v>1783044.35357143</v>
+        <v>1084212.80357143</v>
       </c>
       <c r="F19" s="3"/>
     </row>
@@ -3659,15 +3659,15 @@
       </c>
       <c r="C21" s="18" t="n">
         <f aca="false">IF(C20=0,0,C19/C20)</f>
-        <v>1.1155430625</v>
+        <v>0.5395396875</v>
       </c>
       <c r="D21" s="18" t="n">
         <f aca="false">IF(D20=0,0,D19/D20)</f>
-        <v>4.07765873777778</v>
+        <v>2.26546417777778</v>
       </c>
       <c r="E21" s="18" t="n">
         <f aca="false">IF(E20=0,0,E19/E20)</f>
-        <v>17.8304435357143</v>
+        <v>10.8421280357143</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>46</v>
@@ -3680,15 +3680,15 @@
       </c>
       <c r="C22" s="16" t="n">
         <f aca="false">IF(C16=0,0,C20/C16)</f>
-        <v>14.940406360751</v>
+        <v>30.8905295621403</v>
       </c>
       <c r="D22" s="16" t="n">
         <f aca="false">IF(D16=0,0,D20/D16)</f>
-        <v>5.44975037178633</v>
+        <v>9.80912540582314</v>
       </c>
       <c r="E22" s="16" t="n">
         <f aca="false">IF(E16=0,0,E20/E16)</f>
-        <v>1.60239584137098</v>
+        <v>2.63522331384701</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>48</v>
@@ -3701,15 +3701,15 @@
       </c>
       <c r="C23" s="19" t="n">
         <f aca="false">IF(C16=0,0,(Допущения!$D$18+Допущения!$C$15+Допущения!$D$19)/C16)</f>
-        <v>34.3629346297273</v>
+        <v>71.0482179929226</v>
       </c>
       <c r="D23" s="19" t="n">
         <f aca="false">IF(D16=0,0,(Допущения!$D$18+Допущения!$C$15+Допущения!$D$19)/D16)</f>
-        <v>16.7125678068114</v>
+        <v>30.081317911191</v>
       </c>
       <c r="E23" s="19" t="n">
         <f aca="false">IF(E16=0,0,(Допущения!$D$18+Допущения!$C$15+Допущения!$D$19)/E16)</f>
-        <v>7.37102087030649</v>
+        <v>12.1220272436962</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>50</v>
@@ -3844,7 +3844,7 @@
         <v>58</v>
       </c>
       <c r="C6" s="21" t="n">
-        <v>0.07</v>
+        <v>0.05</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -6467,147 +6467,147 @@
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">C16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>32999.4</v>
+        <v>23571</v>
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">D16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>48014.127</v>
+        <v>34295.805</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">E16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>69882.82938</v>
+        <v>49916.3067</v>
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">F16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>150732.349362</v>
+        <v>107665.96383</v>
       </c>
       <c r="G17" s="12" t="n">
         <f aca="false">G16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>201231.424240308</v>
+        <v>143736.73160022</v>
       </c>
       <c r="H17" s="12" t="n">
         <f aca="false">H16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>255852.778675516</v>
+        <v>182751.984768226</v>
       </c>
       <c r="I17" s="12" t="n">
         <f aca="false">I16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>314167.437951234</v>
+        <v>224405.31282231</v>
       </c>
       <c r="J17" s="12" t="n">
         <f aca="false">J16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>214733.179491791</v>
+        <v>153380.842494136</v>
       </c>
       <c r="K17" s="12" t="n">
         <f aca="false">K16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>264204.662312569</v>
+        <v>188717.615937549</v>
       </c>
       <c r="L17" s="12" t="n">
         <f aca="false">L16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>317196.341748683</v>
+        <v>226568.815534773</v>
       </c>
       <c r="M17" s="12" t="n">
         <f aca="false">M16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>339413.811243762</v>
+        <v>242438.436602687</v>
       </c>
       <c r="N17" s="12" t="n">
         <f aca="false">N16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>360298.232569136</v>
+        <v>257355.880406526</v>
       </c>
       <c r="O17" s="12" t="n">
         <f aca="false">O16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>336943.07089199</v>
+        <v>240673.622065707</v>
       </c>
       <c r="P17" s="12" t="n">
         <f aca="false">P16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>287043.964978853</v>
+        <v>205031.403556324</v>
       </c>
       <c r="Q17" s="12" t="n">
         <f aca="false">Q16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>319320.427080122</v>
+        <v>228086.019342944</v>
       </c>
       <c r="R17" s="12" t="n">
         <f aca="false">R16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>582767.169092191</v>
+        <v>416262.263637279</v>
       </c>
       <c r="S17" s="12" t="n">
         <f aca="false">S16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>693329.602841326</v>
+        <v>495235.430600947</v>
       </c>
       <c r="T17" s="12" t="n">
         <f aca="false">T16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>809976.192731832</v>
+        <v>578554.42337988</v>
       </c>
       <c r="U17" s="12" t="n">
         <f aca="false">U16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>932073.806265249</v>
+        <v>665767.004475178</v>
       </c>
       <c r="V17" s="12" t="n">
         <f aca="false">V16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>605167.647931898</v>
+        <v>432262.605665641</v>
       </c>
       <c r="W17" s="12" t="n">
         <f aca="false">W16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>714213.437687982</v>
+        <v>510152.455491416</v>
       </c>
       <c r="X17" s="12" t="n">
         <f aca="false">X16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>828454.757140781</v>
+        <v>591753.397957701</v>
       </c>
       <c r="Y17" s="12" t="n">
         <f aca="false">Y16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>861245.971712334</v>
+        <v>615175.694080239</v>
       </c>
       <c r="Z17" s="12" t="n">
         <f aca="false">Z16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>892069.713409595</v>
+        <v>637192.652435425</v>
       </c>
       <c r="AA17" s="12" t="n">
         <f aca="false">AA16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>758834.824484015</v>
+        <v>542024.874631439</v>
       </c>
       <c r="AB17" s="12" t="n">
         <f aca="false">AB16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>600977.351261231</v>
+        <v>429269.536615165</v>
       </c>
       <c r="AC17" s="12" t="n">
         <f aca="false">AC16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>630917.510185557</v>
+        <v>450655.364418255</v>
       </c>
       <c r="AD17" s="12" t="n">
         <f aca="false">AD16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1098435.43262404</v>
+        <v>784596.737588599</v>
       </c>
       <c r="AE17" s="12" t="n">
         <f aca="false">AE16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1256780.03733326</v>
+        <v>897700.026666612</v>
       </c>
       <c r="AF17" s="12" t="n">
         <f aca="false">AF16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1420768.40191992</v>
+        <v>1014834.57279994</v>
       </c>
       <c r="AG17" s="12" t="n">
         <f aca="false">AG16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1589813.22262179</v>
+        <v>1135580.87330128</v>
       </c>
       <c r="AH17" s="12" t="n">
         <f aca="false">AH16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1007644.20262429</v>
+        <v>719745.859017353</v>
       </c>
       <c r="AI17" s="12" t="n">
         <f aca="false">AI16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1164581.94427519</v>
+        <v>831844.245910851</v>
       </c>
       <c r="AJ17" s="12" t="n">
         <f aca="false">AJ16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1326339.14179853</v>
+        <v>947385.101284667</v>
       </c>
       <c r="AK17" s="12" t="n">
         <f aca="false">AK16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1356756.79329062</v>
+        <v>969111.995207587</v>
       </c>
       <c r="AL17" s="12" t="n">
         <f aca="false">AL16*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1385349.38569318</v>
+        <v>989535.275495132</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6619,147 +6619,147 @@
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">C16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>13000.5</v>
+        <v>12757.5</v>
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">D16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>18915.7275</v>
+        <v>18562.1625</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">E16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>27531.15885</v>
+        <v>27016.55775</v>
       </c>
       <c r="F18" s="12" t="n">
         <f aca="false">F16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>59382.773865</v>
+        <v>58272.815475</v>
       </c>
       <c r="G18" s="12" t="n">
         <f aca="false">G16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>79277.47567641</v>
+        <v>77795.65370115</v>
       </c>
       <c r="H18" s="12" t="n">
         <f aca="false">H16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>100796.197784537</v>
+        <v>98912.156704452</v>
       </c>
       <c r="I18" s="12" t="n">
         <f aca="false">I16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>123769.940577253</v>
+        <v>121456.483744034</v>
       </c>
       <c r="J18" s="12" t="n">
         <f aca="false">J16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>84596.6502416112</v>
+        <v>83015.4044427025</v>
       </c>
       <c r="K18" s="12" t="n">
         <f aca="false">K16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>104086.520130504</v>
+        <v>102140.977698158</v>
       </c>
       <c r="L18" s="12" t="n">
         <f aca="false">L16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>124963.21269186</v>
+        <v>122627.451706965</v>
       </c>
       <c r="M18" s="12" t="n">
         <f aca="false">M16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>133716.044930348</v>
+        <v>131216.679604547</v>
       </c>
       <c r="N18" s="12" t="n">
         <f aca="false">N16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>141943.707234527</v>
+        <v>139290.553828274</v>
       </c>
       <c r="O18" s="12" t="n">
         <f aca="false">O16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>132742.667840364</v>
+        <v>130261.496478862</v>
       </c>
       <c r="P18" s="12" t="n">
         <f aca="false">P16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>113084.330827457</v>
+        <v>110970.605017598</v>
       </c>
       <c r="Q18" s="12" t="n">
         <f aca="false">Q16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>125800.02097781</v>
+        <v>123448.618716542</v>
       </c>
       <c r="R18" s="12" t="n">
         <f aca="false">R16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>229587.949531902</v>
+        <v>225296.585989249</v>
       </c>
       <c r="S18" s="12" t="n">
         <f aca="false">S16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>273145.314815986</v>
+        <v>268039.794912884</v>
       </c>
       <c r="T18" s="12" t="n">
         <f aca="false">T16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>319099.604647666</v>
+        <v>313135.126056121</v>
       </c>
       <c r="U18" s="12" t="n">
         <f aca="false">U16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>367201.389066206</v>
+        <v>360337.811700483</v>
       </c>
       <c r="V18" s="12" t="n">
         <f aca="false">V16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>238412.880444452</v>
+        <v>233956.564922126</v>
       </c>
       <c r="W18" s="12" t="n">
         <f aca="false">W16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>281372.746070008</v>
+        <v>276113.442405148</v>
       </c>
       <c r="X18" s="12" t="n">
         <f aca="false">X16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>326379.451450897</v>
+        <v>320278.900956488</v>
       </c>
       <c r="Y18" s="12" t="n">
         <f aca="false">Y16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>339297.934363843</v>
+        <v>332955.916899098</v>
       </c>
       <c r="Z18" s="12" t="n">
         <f aca="false">Z16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>351441.308302013</v>
+        <v>344872.311885153</v>
       </c>
       <c r="AA18" s="12" t="n">
         <f aca="false">AA16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>298951.863843113</v>
+        <v>293363.978537635</v>
       </c>
       <c r="AB18" s="12" t="n">
         <f aca="false">AB16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>236762.064009395</v>
+        <v>232336.604869032</v>
       </c>
       <c r="AC18" s="12" t="n">
         <f aca="false">AC16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>248557.340168831</v>
+        <v>243911.408576891</v>
       </c>
       <c r="AD18" s="12" t="n">
         <f aca="false">AD16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>432741.499597836</v>
+        <v>424652.873437129</v>
       </c>
       <c r="AE18" s="12" t="n">
         <f aca="false">AE16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>495123.210584162</v>
+        <v>485868.571133991</v>
       </c>
       <c r="AF18" s="12" t="n">
         <f aca="false">AF16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>559728.346853577</v>
+        <v>549266.134762856</v>
       </c>
       <c r="AG18" s="12" t="n">
         <f aca="false">AG16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>626325.533212559</v>
+        <v>614618.513900175</v>
       </c>
       <c r="AH18" s="12" t="n">
         <f aca="false">AH16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>396973.231519881</v>
+        <v>389553.17111764</v>
       </c>
       <c r="AI18" s="12" t="n">
         <f aca="false">AI16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>458800.692332274</v>
+        <v>450224.978456904</v>
       </c>
       <c r="AJ18" s="12" t="n">
         <f aca="false">AJ16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>522526.834213708</v>
+        <v>512759.977499433</v>
       </c>
       <c r="AK18" s="12" t="n">
         <f aca="false">AK16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>534510.224160886</v>
+        <v>524519.378849467</v>
       </c>
       <c r="AL18" s="12" t="n">
         <f aca="false">AL16*(1+Допущения!$C$6)*Допущения!$C$23</f>
-        <v>545774.610711233</v>
+        <v>535573.216118499</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6923,147 +6923,147 @@
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">C17*Допущения!$C$8</f>
-        <v>1319.976</v>
+        <v>942.84</v>
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">D17*Допущения!$C$8</f>
-        <v>1920.56508</v>
+        <v>1371.8322</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">E17*Допущения!$C$8</f>
-        <v>2795.3131752</v>
+        <v>1996.652268</v>
       </c>
       <c r="F20" s="12" t="n">
         <f aca="false">F17*Допущения!$C$8</f>
-        <v>6029.29397448</v>
+        <v>4306.6385532</v>
       </c>
       <c r="G20" s="12" t="n">
         <f aca="false">G17*Допущения!$C$8</f>
-        <v>8049.25696961232</v>
+        <v>5749.4692640088</v>
       </c>
       <c r="H20" s="12" t="n">
         <f aca="false">H17*Допущения!$C$8</f>
-        <v>10234.1111470206</v>
+        <v>7310.07939072903</v>
       </c>
       <c r="I20" s="12" t="n">
         <f aca="false">I17*Допущения!$C$8</f>
-        <v>12566.6975180493</v>
+        <v>8976.21251289239</v>
       </c>
       <c r="J20" s="12" t="n">
         <f aca="false">J17*Допущения!$C$8</f>
-        <v>8589.32717967162</v>
+        <v>6135.23369976544</v>
       </c>
       <c r="K20" s="12" t="n">
         <f aca="false">K17*Допущения!$C$8</f>
-        <v>10568.1864925027</v>
+        <v>7548.70463750196</v>
       </c>
       <c r="L20" s="12" t="n">
         <f aca="false">L17*Допущения!$C$8</f>
-        <v>12687.8536699473</v>
+        <v>9062.75262139093</v>
       </c>
       <c r="M20" s="12" t="n">
         <f aca="false">M17*Допущения!$C$8</f>
-        <v>13576.5524497505</v>
+        <v>9697.53746410748</v>
       </c>
       <c r="N20" s="12" t="n">
         <f aca="false">N17*Допущения!$C$8</f>
-        <v>14411.9293027654</v>
+        <v>10294.235216261</v>
       </c>
       <c r="O20" s="12" t="n">
         <f aca="false">O17*Допущения!$C$8</f>
-        <v>13477.7228356796</v>
+        <v>9626.9448826283</v>
       </c>
       <c r="P20" s="12" t="n">
         <f aca="false">P17*Допущения!$C$8</f>
-        <v>11481.7585991541</v>
+        <v>8201.25614225295</v>
       </c>
       <c r="Q20" s="12" t="n">
         <f aca="false">Q17*Допущения!$C$8</f>
-        <v>12772.8170832049</v>
+        <v>9123.44077371777</v>
       </c>
       <c r="R20" s="12" t="n">
         <f aca="false">R17*Допущения!$C$8</f>
-        <v>23310.6867636877</v>
+        <v>16650.4905454912</v>
       </c>
       <c r="S20" s="12" t="n">
         <f aca="false">S17*Допущения!$C$8</f>
-        <v>27733.184113653</v>
+        <v>19809.4172240379</v>
       </c>
       <c r="T20" s="12" t="n">
         <f aca="false">T17*Допущения!$C$8</f>
-        <v>32399.0477092733</v>
+        <v>23142.1769351952</v>
       </c>
       <c r="U20" s="12" t="n">
         <f aca="false">U17*Допущения!$C$8</f>
-        <v>37282.95225061</v>
+        <v>26630.6801790071</v>
       </c>
       <c r="V20" s="12" t="n">
         <f aca="false">V17*Допущения!$C$8</f>
-        <v>24206.7059172759</v>
+        <v>17290.5042266257</v>
       </c>
       <c r="W20" s="12" t="n">
         <f aca="false">W17*Допущения!$C$8</f>
-        <v>28568.5375075193</v>
+        <v>20406.0982196566</v>
       </c>
       <c r="X20" s="12" t="n">
         <f aca="false">X17*Допущения!$C$8</f>
-        <v>33138.1902856313</v>
+        <v>23670.135918308</v>
       </c>
       <c r="Y20" s="12" t="n">
         <f aca="false">Y17*Допущения!$C$8</f>
-        <v>34449.8388684934</v>
+        <v>24607.0277632096</v>
       </c>
       <c r="Z20" s="12" t="n">
         <f aca="false">Z17*Допущения!$C$8</f>
-        <v>35682.7885363838</v>
+        <v>25487.706097417</v>
       </c>
       <c r="AA20" s="12" t="n">
         <f aca="false">AA17*Допущения!$C$8</f>
-        <v>30353.3929793606</v>
+        <v>21680.9949852576</v>
       </c>
       <c r="AB20" s="12" t="n">
         <f aca="false">AB17*Допущения!$C$8</f>
-        <v>24039.0940504492</v>
+        <v>17170.7814646066</v>
       </c>
       <c r="AC20" s="12" t="n">
         <f aca="false">AC17*Допущения!$C$8</f>
-        <v>25236.7004074223</v>
+        <v>18026.2145767302</v>
       </c>
       <c r="AD20" s="12" t="n">
         <f aca="false">AD17*Допущения!$C$8</f>
-        <v>43937.4173049616</v>
+        <v>31383.869503544</v>
       </c>
       <c r="AE20" s="12" t="n">
         <f aca="false">AE17*Допущения!$C$8</f>
-        <v>50271.2014933303</v>
+        <v>35908.0010666645</v>
       </c>
       <c r="AF20" s="12" t="n">
         <f aca="false">AF17*Допущения!$C$8</f>
-        <v>56830.7360767968</v>
+        <v>40593.3829119977</v>
       </c>
       <c r="AG20" s="12" t="n">
         <f aca="false">AG17*Допущения!$C$8</f>
-        <v>63592.5289048715</v>
+        <v>45423.234932051</v>
       </c>
       <c r="AH20" s="12" t="n">
         <f aca="false">AH17*Допущения!$C$8</f>
-        <v>40305.7681049718</v>
+        <v>28789.8343606941</v>
       </c>
       <c r="AI20" s="12" t="n">
         <f aca="false">AI17*Допущения!$C$8</f>
-        <v>46583.2777710077</v>
+        <v>33273.7698364341</v>
       </c>
       <c r="AJ20" s="12" t="n">
         <f aca="false">AJ17*Допущения!$C$8</f>
-        <v>53053.5656719413</v>
+        <v>37895.4040513867</v>
       </c>
       <c r="AK20" s="12" t="n">
         <f aca="false">AK17*Допущения!$C$8</f>
-        <v>54270.2717316249</v>
+        <v>38764.4798083035</v>
       </c>
       <c r="AL20" s="12" t="n">
         <f aca="false">AL17*Допущения!$C$8</f>
-        <v>55413.9754277274</v>
+        <v>39581.4110198053</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7075,147 +7075,147 @@
       </c>
       <c r="C21" s="33" t="n">
         <f aca="false">C17-C18-C19-C20</f>
-        <v>17058.924</v>
+        <v>8250.66</v>
       </c>
       <c r="D21" s="33" t="n">
         <f aca="false">D17-D18-D19-D20</f>
-        <v>24820.73442</v>
+        <v>12004.7103</v>
       </c>
       <c r="E21" s="33" t="n">
         <f aca="false">E17-E18-E19-E20</f>
-        <v>36125.6833548</v>
+        <v>17472.422682</v>
       </c>
       <c r="F21" s="33" t="n">
         <f aca="false">F17-F18-F19-F20</f>
-        <v>77920.55892252</v>
+        <v>37686.7872018</v>
       </c>
       <c r="G21" s="33" t="n">
         <f aca="false">G17-G18-G19-G20</f>
-        <v>104025.878425886</v>
+        <v>50312.7954666612</v>
       </c>
       <c r="H21" s="33" t="n">
         <f aca="false">H17-H18-H19-H20</f>
-        <v>132262.195876726</v>
+        <v>63969.4748058126</v>
       </c>
       <c r="I21" s="33" t="n">
         <f aca="false">I17-I18-I19-I20</f>
-        <v>162407.754301133</v>
+        <v>78549.5710105858</v>
       </c>
       <c r="J21" s="33" t="n">
         <f aca="false">J17-J18-J19-J20</f>
-        <v>111005.563411117</v>
+        <v>53688.5656922773</v>
       </c>
       <c r="K21" s="33" t="n">
         <f aca="false">K17-K18-K19-K20</f>
-        <v>136579.672807256</v>
+        <v>66057.6507195833</v>
       </c>
       <c r="L21" s="33" t="n">
         <f aca="false">L17-L18-L19-L20</f>
-        <v>163973.535487579</v>
+        <v>79306.8713071203</v>
       </c>
       <c r="M21" s="33" t="n">
         <f aca="false">M17-M18-M19-M20</f>
-        <v>175458.778358324</v>
+        <v>84861.7840286931</v>
       </c>
       <c r="N21" s="33" t="n">
         <f aca="false">N17-N18-N19-N20</f>
-        <v>186254.906656825</v>
+        <v>90083.4019869715</v>
       </c>
       <c r="O21" s="33" t="n">
         <f aca="false">O17-O18-O19-O20</f>
-        <v>174181.537805932</v>
+        <v>84244.0382942026</v>
       </c>
       <c r="P21" s="33" t="n">
         <f aca="false">P17-P18-P19-P20</f>
-        <v>148386.370153182</v>
+        <v>71768.0369974128</v>
       </c>
       <c r="Q21" s="33" t="n">
         <f aca="false">Q17-Q18-Q19-Q20</f>
-        <v>165071.573943991</v>
+        <v>79837.9447775681</v>
       </c>
       <c r="R21" s="33" t="n">
         <f aca="false">R17-R18-R19-R20</f>
-        <v>301259.442512253</v>
+        <v>145706.09681819</v>
       </c>
       <c r="S21" s="33" t="n">
         <f aca="false">S17-S18-S19-S20</f>
-        <v>358414.30455767</v>
+        <v>173349.419110008</v>
       </c>
       <c r="T21" s="33" t="n">
         <f aca="false">T17-T18-T19-T20</f>
-        <v>418714.349764592</v>
+        <v>202513.929778263</v>
       </c>
       <c r="U21" s="33" t="n">
         <f aca="false">U17-U18-U19-U20</f>
-        <v>481832.282510276</v>
+        <v>233041.330157531</v>
       </c>
       <c r="V21" s="33" t="n">
         <f aca="false">V17-V18-V19-V20</f>
-        <v>312839.291421329</v>
+        <v>151306.766368049</v>
       </c>
       <c r="W21" s="33" t="n">
         <f aca="false">W17-W18-W19-W20</f>
-        <v>369210.129678055</v>
+        <v>178570.890434212</v>
       </c>
       <c r="X21" s="33" t="n">
         <f aca="false">X17-X18-X19-X20</f>
-        <v>428266.778774858</v>
+        <v>207134.02445351</v>
       </c>
       <c r="Y21" s="33" t="n">
         <f aca="false">Y17-Y18-Y19-Y20</f>
-        <v>445218.082048366</v>
+        <v>215332.632986299</v>
       </c>
       <c r="Z21" s="33" t="n">
         <f aca="false">Z17-Z18-Z19-Z20</f>
-        <v>461152.307125465</v>
+        <v>223039.325007121</v>
       </c>
       <c r="AA21" s="33" t="n">
         <f aca="false">AA17-AA18-AA19-AA20</f>
-        <v>392276.998958349</v>
+        <v>189727.332405355</v>
       </c>
       <c r="AB21" s="33" t="n">
         <f aca="false">AB17-AB18-AB19-AB20</f>
-        <v>310673.132265636</v>
+        <v>150259.089345776</v>
       </c>
       <c r="AC21" s="33" t="n">
         <f aca="false">AC17-AC18-AC19-AC20</f>
-        <v>326150.592329698</v>
+        <v>157744.863985029</v>
       </c>
       <c r="AD21" s="33" t="n">
         <f aca="false">AD17-AD18-AD19-AD20</f>
-        <v>567832.341316527</v>
+        <v>274635.820243212</v>
       </c>
       <c r="AE21" s="33" t="n">
         <f aca="false">AE17-AE18-AE19-AE20</f>
-        <v>649688.028921289</v>
+        <v>314225.858131481</v>
       </c>
       <c r="AF21" s="33" t="n">
         <f aca="false">AF17-AF18-AF19-AF20</f>
-        <v>734461.23838474</v>
+        <v>355226.974520282</v>
       </c>
       <c r="AG21" s="33" t="n">
         <f aca="false">AG17-AG18-AG19-AG20</f>
-        <v>821848.36508846</v>
+        <v>397492.329053154</v>
       </c>
       <c r="AH21" s="33" t="n">
         <f aca="false">AH17-AH18-AH19-AH20</f>
-        <v>520898.133651171</v>
+        <v>251935.784190748</v>
       </c>
       <c r="AI21" s="33" t="n">
         <f aca="false">AI17-AI18-AI19-AI20</f>
-        <v>602026.548336113</v>
+        <v>291174.071781716</v>
       </c>
       <c r="AJ21" s="33" t="n">
         <f aca="false">AJ17-AJ18-AJ19-AJ20</f>
-        <v>685646.363817718</v>
+        <v>331617.341638681</v>
       </c>
       <c r="AK21" s="33" t="n">
         <f aca="false">AK17-AK18-AK19-AK20</f>
-        <v>701370.661988655</v>
+        <v>339222.50114036</v>
       </c>
       <c r="AL21" s="33" t="n">
         <f aca="false">AL17-AL18-AL19-AL20</f>
-        <v>716151.502269336</v>
+        <v>346371.351071939</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7987,147 +7987,147 @@
       </c>
       <c r="C27" s="33" t="n">
         <f aca="false">C21-C26</f>
-        <v>-1182941.076</v>
+        <v>-1191749.34</v>
       </c>
       <c r="D27" s="33" t="n">
         <f aca="false">D21-D26</f>
-        <v>-375179.26558</v>
+        <v>-387995.2897</v>
       </c>
       <c r="E27" s="33" t="n">
         <f aca="false">E21-E26</f>
-        <v>-363874.3166452</v>
+        <v>-382527.577318</v>
       </c>
       <c r="F27" s="33" t="n">
         <f aca="false">F21-F26</f>
-        <v>-322079.44107748</v>
+        <v>-362313.2127982</v>
       </c>
       <c r="G27" s="33" t="n">
         <f aca="false">G21-G26</f>
-        <v>-295974.121574114</v>
+        <v>-349687.204533339</v>
       </c>
       <c r="H27" s="33" t="n">
         <f aca="false">H21-H26</f>
-        <v>-267737.804123274</v>
+        <v>-336030.525194187</v>
       </c>
       <c r="I27" s="33" t="n">
         <f aca="false">I21-I26</f>
-        <v>-237592.245698867</v>
+        <v>-321450.428989414</v>
       </c>
       <c r="J27" s="33" t="n">
         <f aca="false">J21-J26</f>
-        <v>-288994.436588883</v>
+        <v>-346311.434307723</v>
       </c>
       <c r="K27" s="33" t="n">
         <f aca="false">K21-K26</f>
-        <v>-263420.327192744</v>
+        <v>-333942.349280417</v>
       </c>
       <c r="L27" s="33" t="n">
         <f aca="false">L21-L26</f>
-        <v>-236026.464512421</v>
+        <v>-320693.12869288</v>
       </c>
       <c r="M27" s="33" t="n">
         <f aca="false">M21-M26</f>
-        <v>-224541.221641676</v>
+        <v>-315138.215971307</v>
       </c>
       <c r="N27" s="33" t="n">
         <f aca="false">N21-N26</f>
-        <v>-213745.093343175</v>
+        <v>-309916.598013028</v>
       </c>
       <c r="O27" s="33" t="n">
         <f aca="false">O21-O26</f>
-        <v>-885818.462194068</v>
+        <v>-975755.961705797</v>
       </c>
       <c r="P27" s="33" t="n">
         <f aca="false">P21-P26</f>
-        <v>-911613.629846818</v>
+        <v>-988231.963002587</v>
       </c>
       <c r="Q27" s="33" t="n">
         <f aca="false">Q21-Q26</f>
-        <v>-894928.426056009</v>
+        <v>-980162.055222432</v>
       </c>
       <c r="R27" s="33" t="n">
         <f aca="false">R21-R26</f>
-        <v>-758740.557487747</v>
+        <v>-914293.90318181</v>
       </c>
       <c r="S27" s="33" t="n">
         <f aca="false">S21-S26</f>
-        <v>-701585.69544233</v>
+        <v>-886650.580889992</v>
       </c>
       <c r="T27" s="33" t="n">
         <f aca="false">T21-T26</f>
-        <v>-641285.650235408</v>
+        <v>-857486.070221737</v>
       </c>
       <c r="U27" s="33" t="n">
         <f aca="false">U21-U26</f>
-        <v>-578167.717489724</v>
+        <v>-826958.669842469</v>
       </c>
       <c r="V27" s="33" t="n">
         <f aca="false">V21-V26</f>
-        <v>-747160.708578671</v>
+        <v>-908693.233631951</v>
       </c>
       <c r="W27" s="33" t="n">
         <f aca="false">W21-W26</f>
-        <v>-690789.870321945</v>
+        <v>-881429.109565788</v>
       </c>
       <c r="X27" s="33" t="n">
         <f aca="false">X21-X26</f>
-        <v>-631733.221225142</v>
+        <v>-852865.97554649</v>
       </c>
       <c r="Y27" s="33" t="n">
         <f aca="false">Y21-Y26</f>
-        <v>-614781.917951634</v>
+        <v>-844667.367013701</v>
       </c>
       <c r="Z27" s="33" t="n">
         <f aca="false">Z21-Z26</f>
-        <v>-598847.692874536</v>
+        <v>-836960.674992879</v>
       </c>
       <c r="AA27" s="33" t="n">
         <f aca="false">AA21-AA26</f>
-        <v>-1147723.00104165</v>
+        <v>-1350272.66759464</v>
       </c>
       <c r="AB27" s="33" t="n">
         <f aca="false">AB21-AB26</f>
-        <v>-1229326.86773436</v>
+        <v>-1389740.91065422</v>
       </c>
       <c r="AC27" s="33" t="n">
         <f aca="false">AC21-AC26</f>
-        <v>-1213849.4076703</v>
+        <v>-1382255.13601497</v>
       </c>
       <c r="AD27" s="33" t="n">
         <f aca="false">AD21-AD26</f>
-        <v>-972167.658683473</v>
+        <v>-1265364.17975679</v>
       </c>
       <c r="AE27" s="33" t="n">
         <f aca="false">AE21-AE26</f>
-        <v>-890311.971078711</v>
+        <v>-1225774.14186852</v>
       </c>
       <c r="AF27" s="33" t="n">
         <f aca="false">AF21-AF26</f>
-        <v>-805538.76161526</v>
+        <v>-1184773.02547972</v>
       </c>
       <c r="AG27" s="33" t="n">
         <f aca="false">AG21-AG26</f>
-        <v>-718151.63491154</v>
+        <v>-1142507.67094685</v>
       </c>
       <c r="AH27" s="33" t="n">
         <f aca="false">AH21-AH26</f>
-        <v>-1019101.86634883</v>
+        <v>-1288064.21580925</v>
       </c>
       <c r="AI27" s="33" t="n">
         <f aca="false">AI21-AI26</f>
-        <v>-937973.451663887</v>
+        <v>-1248825.92821828</v>
       </c>
       <c r="AJ27" s="33" t="n">
         <f aca="false">AJ21-AJ26</f>
-        <v>-854353.636182282</v>
+        <v>-1208382.65836132</v>
       </c>
       <c r="AK27" s="33" t="n">
         <f aca="false">AK21-AK26</f>
-        <v>-838629.338011345</v>
+        <v>-1200777.49885964</v>
       </c>
       <c r="AL27" s="33" t="n">
         <f aca="false">AL21-AL26</f>
-        <v>-823848.497730664</v>
+        <v>-1193628.64892806</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8139,147 +8139,147 @@
       </c>
       <c r="C28" s="33" t="n">
         <f aca="false">C27</f>
-        <v>-1182941.076</v>
+        <v>-1191749.34</v>
       </c>
       <c r="D28" s="33" t="n">
         <f aca="false">C28+D27</f>
-        <v>-1558120.34158</v>
+        <v>-1579744.6297</v>
       </c>
       <c r="E28" s="33" t="n">
         <f aca="false">D28+E27</f>
-        <v>-1921994.6582252</v>
+        <v>-1962272.207018</v>
       </c>
       <c r="F28" s="33" t="n">
         <f aca="false">E28+F27</f>
-        <v>-2244074.09930268</v>
+        <v>-2324585.4198162</v>
       </c>
       <c r="G28" s="33" t="n">
         <f aca="false">F28+G27</f>
-        <v>-2540048.22087679</v>
+        <v>-2674272.62434954</v>
       </c>
       <c r="H28" s="33" t="n">
         <f aca="false">G28+H27</f>
-        <v>-2807786.02500007</v>
+        <v>-3010303.14954373</v>
       </c>
       <c r="I28" s="33" t="n">
         <f aca="false">H28+I27</f>
-        <v>-3045378.27069894</v>
+        <v>-3331753.57853314</v>
       </c>
       <c r="J28" s="33" t="n">
         <f aca="false">I28+J27</f>
-        <v>-3334372.70728782</v>
+        <v>-3678065.01284086</v>
       </c>
       <c r="K28" s="33" t="n">
         <f aca="false">J28+K27</f>
-        <v>-3597793.03448056</v>
+        <v>-4012007.36212128</v>
       </c>
       <c r="L28" s="33" t="n">
         <f aca="false">K28+L27</f>
-        <v>-3833819.49899298</v>
+        <v>-4332700.49081416</v>
       </c>
       <c r="M28" s="33" t="n">
         <f aca="false">L28+M27</f>
-        <v>-4058360.72063466</v>
+        <v>-4647838.70678547</v>
       </c>
       <c r="N28" s="33" t="n">
         <f aca="false">M28+N27</f>
-        <v>-4272105.81397783</v>
+        <v>-4957755.3047985</v>
       </c>
       <c r="O28" s="33" t="n">
         <f aca="false">N28+O27</f>
-        <v>-5157924.2761719</v>
+        <v>-5933511.26650429</v>
       </c>
       <c r="P28" s="33" t="n">
         <f aca="false">O28+P27</f>
-        <v>-6069537.90601872</v>
+        <v>-6921743.22950688</v>
       </c>
       <c r="Q28" s="33" t="n">
         <f aca="false">P28+Q27</f>
-        <v>-6964466.33207473</v>
+        <v>-7901905.28472931</v>
       </c>
       <c r="R28" s="33" t="n">
         <f aca="false">Q28+R27</f>
-        <v>-7723206.88956248</v>
+        <v>-8816199.18791112</v>
       </c>
       <c r="S28" s="33" t="n">
         <f aca="false">R28+S27</f>
-        <v>-8424792.58500481</v>
+        <v>-9702849.76880112</v>
       </c>
       <c r="T28" s="33" t="n">
         <f aca="false">S28+T27</f>
-        <v>-9066078.23524021</v>
+        <v>-10560335.8390229</v>
       </c>
       <c r="U28" s="33" t="n">
         <f aca="false">T28+U27</f>
-        <v>-9644245.95272994</v>
+        <v>-11387294.5088653</v>
       </c>
       <c r="V28" s="33" t="n">
         <f aca="false">U28+V27</f>
-        <v>-10391406.6613086</v>
+        <v>-12295987.7424973</v>
       </c>
       <c r="W28" s="33" t="n">
         <f aca="false">V28+W27</f>
-        <v>-11082196.5316306</v>
+        <v>-13177416.8520631</v>
       </c>
       <c r="X28" s="33" t="n">
         <f aca="false">W28+X27</f>
-        <v>-11713929.7528557</v>
+        <v>-14030282.8276096</v>
       </c>
       <c r="Y28" s="33" t="n">
         <f aca="false">X28+Y27</f>
-        <v>-12328711.6708073</v>
+        <v>-14874950.1946233</v>
       </c>
       <c r="Z28" s="33" t="n">
         <f aca="false">Y28+Z27</f>
-        <v>-12927559.3636819</v>
+        <v>-15711910.8696161</v>
       </c>
       <c r="AA28" s="33" t="n">
         <f aca="false">Z28+AA27</f>
-        <v>-14075282.3647235</v>
+        <v>-17062183.5372108</v>
       </c>
       <c r="AB28" s="33" t="n">
         <f aca="false">AA28+AB27</f>
-        <v>-15304609.2324579</v>
+        <v>-18451924.447865</v>
       </c>
       <c r="AC28" s="33" t="n">
         <f aca="false">AB28+AC27</f>
-        <v>-16518458.6401282</v>
+        <v>-19834179.58388</v>
       </c>
       <c r="AD28" s="33" t="n">
         <f aca="false">AC28+AD27</f>
-        <v>-17490626.2988117</v>
+        <v>-21099543.7636368</v>
       </c>
       <c r="AE28" s="33" t="n">
         <f aca="false">AD28+AE27</f>
-        <v>-18380938.2698904</v>
+        <v>-22325317.9055053</v>
       </c>
       <c r="AF28" s="33" t="n">
         <f aca="false">AE28+AF27</f>
-        <v>-19186477.0315056</v>
+        <v>-23510090.930985</v>
       </c>
       <c r="AG28" s="33" t="n">
         <f aca="false">AF28+AG27</f>
-        <v>-19904628.6664172</v>
+        <v>-24652598.6019318</v>
       </c>
       <c r="AH28" s="33" t="n">
         <f aca="false">AG28+AH27</f>
-        <v>-20923730.532766</v>
+        <v>-25940662.8177411</v>
       </c>
       <c r="AI28" s="33" t="n">
         <f aca="false">AH28+AI27</f>
-        <v>-21861703.9844299</v>
+        <v>-27189488.7459594</v>
       </c>
       <c r="AJ28" s="33" t="n">
         <f aca="false">AI28+AJ27</f>
-        <v>-22716057.6206122</v>
+        <v>-28397871.4043207</v>
       </c>
       <c r="AK28" s="33" t="n">
         <f aca="false">AJ28+AK27</f>
-        <v>-23554686.9586235</v>
+        <v>-29598648.9031803</v>
       </c>
       <c r="AL28" s="33" t="n">
         <f aca="false">AK28+AL27</f>
-        <v>-24378535.4563542</v>
+        <v>-30792277.5521084</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9777,147 +9777,147 @@
       </c>
       <c r="C41" s="12" t="n">
         <f aca="false">C40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>116157.888</v>
+        <v>82969.92</v>
       </c>
       <c r="D41" s="12" t="n">
         <f aca="false">D40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>170316.50328</v>
+        <v>121654.6452</v>
       </c>
       <c r="E41" s="12" t="n">
         <f aca="false">E40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>249770.6766324</v>
+        <v>178407.626166</v>
       </c>
       <c r="F41" s="12" t="n">
         <f aca="false">F40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>542749.02030657</v>
+        <v>387677.87164755</v>
       </c>
       <c r="G41" s="12" t="n">
         <f aca="false">G40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>729874.941832052</v>
+        <v>521339.244165751</v>
       </c>
       <c r="H41" s="12" t="n">
         <f aca="false">H40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>934633.816854119</v>
+        <v>667595.583467228</v>
       </c>
       <c r="I41" s="12" t="n">
         <f aca="false">I40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1155713.13768699</v>
+        <v>825509.384062136</v>
       </c>
       <c r="J41" s="12" t="n">
         <f aca="false">J40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>795361.608917586</v>
+        <v>568115.434941133</v>
       </c>
       <c r="K41" s="12" t="n">
         <f aca="false">K40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>985194.252580831</v>
+        <v>703710.180414879</v>
       </c>
       <c r="L41" s="12" t="n">
         <f aca="false">L40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1190597.92801633</v>
+        <v>850427.091440233</v>
       </c>
       <c r="M41" s="12" t="n">
         <f aca="false">M40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1282218.38125559</v>
+        <v>915870.272325422</v>
       </c>
       <c r="N41" s="12" t="n">
         <f aca="false">N40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1369715.91409909</v>
+        <v>978368.510070779</v>
       </c>
       <c r="O41" s="12" t="n">
         <f aca="false">O40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1240059.4383717</v>
+        <v>885756.741694075</v>
       </c>
       <c r="P41" s="12" t="n">
         <f aca="false">P40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1033389.93273373</v>
+        <v>738135.666238381</v>
       </c>
       <c r="Q41" s="12" t="n">
         <f aca="false">Q40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1132084.74576072</v>
+        <v>808631.961257654</v>
       </c>
       <c r="R41" s="12" t="n">
         <f aca="false">R40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2043897.15366914</v>
+        <v>1459926.5383351</v>
       </c>
       <c r="S41" s="12" t="n">
         <f aca="false">S40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2413309.11992943</v>
+        <v>1723792.22852102</v>
       </c>
       <c r="T41" s="12" t="n">
         <f aca="false">T40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2804624.03949012</v>
+        <v>2003302.88535008</v>
       </c>
       <c r="U41" s="12" t="n">
         <f aca="false">U40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3216211.56752248</v>
+        <v>2297293.97680177</v>
       </c>
       <c r="V41" s="12" t="n">
         <f aca="false">V40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2083739.27814398</v>
+        <v>1488385.19867427</v>
       </c>
       <c r="W41" s="12" t="n">
         <f aca="false">W40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2456513.42695594</v>
+        <v>1754652.44782567</v>
       </c>
       <c r="X41" s="12" t="n">
         <f aca="false">X40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2848629.29193658</v>
+        <v>2034735.20852613</v>
       </c>
       <c r="Y41" s="12" t="n">
         <f aca="false">Y40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2962436.57379944</v>
+        <v>2116026.12414245</v>
       </c>
       <c r="Z41" s="12" t="n">
         <f aca="false">Z40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3071122.52797846</v>
+        <v>2193658.94855604</v>
       </c>
       <c r="AA41" s="12" t="n">
         <f aca="false">AA40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2617372.68337554</v>
+        <v>1869551.91669682</v>
       </c>
       <c r="AB41" s="12" t="n">
         <f aca="false">AB40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2077969.48846773</v>
+        <v>1484263.9203341</v>
       </c>
       <c r="AC41" s="12" t="n">
         <f aca="false">AC40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2187737.16548669</v>
+        <v>1562669.40391906</v>
       </c>
       <c r="AD41" s="12" t="n">
         <f aca="false">AD40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3820942.16173297</v>
+        <v>2729244.40123784</v>
       </c>
       <c r="AE41" s="12" t="n">
         <f aca="false">AE40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4386572.96490049</v>
+        <v>3133266.40350035</v>
       </c>
       <c r="AF41" s="12" t="n">
         <f aca="false">AF40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4976564.07870542</v>
+        <v>3554688.62764673</v>
       </c>
       <c r="AG41" s="12" t="n">
         <f aca="false">AG40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>5589102.24509398</v>
+        <v>3992215.88935284</v>
       </c>
       <c r="AH41" s="12" t="n">
         <f aca="false">AH40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3555707.46834754</v>
+        <v>2539791.04881967</v>
       </c>
       <c r="AI41" s="12" t="n">
         <f aca="false">AI40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4125077.66730589</v>
+        <v>2946484.04807563</v>
       </c>
       <c r="AJ41" s="12" t="n">
         <f aca="false">AJ40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4715959.58697458</v>
+        <v>3368542.5621247</v>
       </c>
       <c r="AK41" s="12" t="n">
         <f aca="false">AK40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4842535.24556072</v>
+        <v>3458953.74682909</v>
       </c>
       <c r="AL41" s="12" t="n">
         <f aca="false">AL40*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4963414.99951049</v>
+        <v>3545296.42822178</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9929,147 +9929,147 @@
       </c>
       <c r="C42" s="12" t="n">
         <f aca="false">C40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>36609.408</v>
+        <v>35925.12</v>
       </c>
       <c r="D42" s="12" t="n">
         <f aca="false">D40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>53678.54448</v>
+        <v>52675.2072</v>
       </c>
       <c r="E42" s="12" t="n">
         <f aca="false">E40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>78720.0659784</v>
+        <v>77248.662876</v>
       </c>
       <c r="F42" s="12" t="n">
         <f aca="false">F40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>171057.86501562</v>
+        <v>167860.5217443</v>
       </c>
       <c r="G42" s="12" t="n">
         <f aca="false">G40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>230034.223198909</v>
+        <v>225734.518092387</v>
       </c>
       <c r="H42" s="12" t="n">
         <f aca="false">H40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>294567.948169045</v>
+        <v>289062.005212614</v>
       </c>
       <c r="I42" s="12" t="n">
         <f aca="false">I40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>364245.377709891</v>
+        <v>357437.052892884</v>
       </c>
       <c r="J42" s="12" t="n">
         <f aca="false">J40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>250673.614592582</v>
+        <v>245988.126469356</v>
       </c>
       <c r="K42" s="12" t="n">
         <f aca="false">K40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>310503.048677905</v>
+        <v>304699.253375515</v>
       </c>
       <c r="L42" s="12" t="n">
         <f aca="false">L40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>375239.994986</v>
+        <v>368226.163304018</v>
       </c>
       <c r="M42" s="12" t="n">
         <f aca="false">M40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>404115.95521163</v>
+        <v>396562.385955338</v>
       </c>
       <c r="N42" s="12" t="n">
         <f aca="false">N40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>431692.497227106</v>
+        <v>423623.478587347</v>
       </c>
       <c r="O42" s="12" t="n">
         <f aca="false">O40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>390828.747881509</v>
+        <v>383523.537640733</v>
       </c>
       <c r="P42" s="12" t="n">
         <f aca="false">P40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>325692.850670131</v>
+        <v>319605.133835175</v>
       </c>
       <c r="Q42" s="12" t="n">
         <f aca="false">Q40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>356798.432389975</v>
+        <v>350129.302812593</v>
       </c>
       <c r="R42" s="12" t="n">
         <f aca="false">R40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>644173.771554044</v>
+        <v>632133.140310043</v>
       </c>
       <c r="S42" s="12" t="n">
         <f aca="false">S40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>760601.107017523</v>
+        <v>746384.2638957</v>
       </c>
       <c r="T42" s="12" t="n">
         <f aca="false">T40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>883931.582401892</v>
+        <v>867409.49674952</v>
       </c>
       <c r="U42" s="12" t="n">
         <f aca="false">U40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1013651.36295996</v>
+        <v>994704.608512108</v>
       </c>
       <c r="V42" s="12" t="n">
         <f aca="false">V40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>656730.788693391</v>
+        <v>644455.446848654</v>
       </c>
       <c r="W42" s="12" t="n">
         <f aca="false">W40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>774217.781102461</v>
+        <v>759746.420708023</v>
       </c>
       <c r="X42" s="12" t="n">
         <f aca="false">X40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>897800.689947612</v>
+        <v>881019.36864018</v>
       </c>
       <c r="Y42" s="12" t="n">
         <f aca="false">Y40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>933669.258899969</v>
+        <v>916217.497051372</v>
       </c>
       <c r="Z42" s="12" t="n">
         <f aca="false">Z40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>967923.742249471</v>
+        <v>949831.70968406</v>
       </c>
       <c r="AA42" s="12" t="n">
         <f aca="false">AA40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>824915.691078596</v>
+        <v>809496.706198622</v>
       </c>
       <c r="AB42" s="12" t="n">
         <f aca="false">AB40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>654912.327735044</v>
+        <v>642670.975814763</v>
       </c>
       <c r="AC42" s="12" t="n">
         <f aca="false">AC40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>689507.736986967</v>
+        <v>676619.741903099</v>
       </c>
       <c r="AD42" s="12" t="n">
         <f aca="false">AD40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1204243.92137092</v>
+        <v>1181734.68919577</v>
       </c>
       <c r="AE42" s="12" t="n">
         <f aca="false">AE40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1382513.42340015</v>
+        <v>1356672.05100015</v>
       </c>
       <c r="AF42" s="12" t="n">
         <f aca="false">AF40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1568460.54910598</v>
+        <v>1539143.52949652</v>
       </c>
       <c r="AG42" s="12" t="n">
         <f aca="false">AG40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1761513.81509589</v>
+        <v>1728588.32322494</v>
       </c>
       <c r="AH42" s="12" t="n">
         <f aca="false">AH40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1120650.07102559</v>
+        <v>1099703.34072604</v>
       </c>
       <c r="AI42" s="12" t="n">
         <f aca="false">AI40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1300098.11605811</v>
+        <v>1275797.21669254</v>
       </c>
       <c r="AJ42" s="12" t="n">
         <f aca="false">AJ40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1486325.99648389</v>
+        <v>1458544.20215709</v>
       </c>
       <c r="AK42" s="12" t="n">
         <f aca="false">AK40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1526218.76664211</v>
+        <v>1497691.31306002</v>
       </c>
       <c r="AL42" s="12" t="n">
         <f aca="false">AL40*(1+Допущения!$C$6)*Допущения!$D$23</f>
-        <v>1564316.36214322</v>
+        <v>1535076.80397232</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10233,147 +10233,147 @@
       </c>
       <c r="C44" s="12" t="n">
         <f aca="false">C41*Допущения!$C$8</f>
-        <v>4646.31552</v>
+        <v>3318.7968</v>
       </c>
       <c r="D44" s="12" t="n">
         <f aca="false">D41*Допущения!$C$8</f>
-        <v>6812.6601312</v>
+        <v>4866.185808</v>
       </c>
       <c r="E44" s="12" t="n">
         <f aca="false">E41*Допущения!$C$8</f>
-        <v>9990.827065296</v>
+        <v>7136.30504664</v>
       </c>
       <c r="F44" s="12" t="n">
         <f aca="false">F41*Допущения!$C$8</f>
-        <v>21709.9608122628</v>
+        <v>15507.114865902</v>
       </c>
       <c r="G44" s="12" t="n">
         <f aca="false">G41*Допущения!$C$8</f>
-        <v>29194.9976732821</v>
+        <v>20853.5697666301</v>
       </c>
       <c r="H44" s="12" t="n">
         <f aca="false">H41*Допущения!$C$8</f>
-        <v>37385.3526741648</v>
+        <v>26703.8233386891</v>
       </c>
       <c r="I44" s="12" t="n">
         <f aca="false">I41*Допущения!$C$8</f>
-        <v>46228.5255074796</v>
+        <v>33020.3753624855</v>
       </c>
       <c r="J44" s="12" t="n">
         <f aca="false">J41*Допущения!$C$8</f>
-        <v>31814.4643567034</v>
+        <v>22724.6173976453</v>
       </c>
       <c r="K44" s="12" t="n">
         <f aca="false">K41*Допущения!$C$8</f>
-        <v>39407.7701032332</v>
+        <v>28148.4072165952</v>
       </c>
       <c r="L44" s="12" t="n">
         <f aca="false">L41*Допущения!$C$8</f>
-        <v>47623.917120653</v>
+        <v>34017.0836576093</v>
       </c>
       <c r="M44" s="12" t="n">
         <f aca="false">M41*Допущения!$C$8</f>
-        <v>51288.7352502237</v>
+        <v>36634.8108930169</v>
       </c>
       <c r="N44" s="12" t="n">
         <f aca="false">N41*Допущения!$C$8</f>
-        <v>54788.6365639636</v>
+        <v>39134.7404028311</v>
       </c>
       <c r="O44" s="12" t="n">
         <f aca="false">O41*Допущения!$C$8</f>
-        <v>49602.3775348682</v>
+        <v>35430.269667763</v>
       </c>
       <c r="P44" s="12" t="n">
         <f aca="false">P41*Допущения!$C$8</f>
-        <v>41335.5973093493</v>
+        <v>29525.4266495352</v>
       </c>
       <c r="Q44" s="12" t="n">
         <f aca="false">Q41*Допущения!$C$8</f>
-        <v>45283.3898304286</v>
+        <v>32345.2784503062</v>
       </c>
       <c r="R44" s="12" t="n">
         <f aca="false">R41*Допущения!$C$8</f>
-        <v>81755.8861467656</v>
+        <v>58397.061533404</v>
       </c>
       <c r="S44" s="12" t="n">
         <f aca="false">S41*Допущения!$C$8</f>
-        <v>96532.3647971772</v>
+        <v>68951.6891408409</v>
       </c>
       <c r="T44" s="12" t="n">
         <f aca="false">T41*Допущения!$C$8</f>
-        <v>112184.961579605</v>
+        <v>80132.1154140033</v>
       </c>
       <c r="U44" s="12" t="n">
         <f aca="false">U41*Допущения!$C$8</f>
-        <v>128648.462700899</v>
+        <v>91891.7590720709</v>
       </c>
       <c r="V44" s="12" t="n">
         <f aca="false">V41*Допущения!$C$8</f>
-        <v>83349.5711257593</v>
+        <v>59535.4079469709</v>
       </c>
       <c r="W44" s="12" t="n">
         <f aca="false">W41*Допущения!$C$8</f>
-        <v>98260.5370782376</v>
+        <v>70186.0979130269</v>
       </c>
       <c r="X44" s="12" t="n">
         <f aca="false">X41*Допущения!$C$8</f>
-        <v>113945.171677463</v>
+        <v>81389.4083410452</v>
       </c>
       <c r="Y44" s="12" t="n">
         <f aca="false">Y41*Допущения!$C$8</f>
-        <v>118497.462951977</v>
+        <v>84641.0449656981</v>
       </c>
       <c r="Z44" s="12" t="n">
         <f aca="false">Z41*Допущения!$C$8</f>
-        <v>122844.901119138</v>
+        <v>87746.3579422418</v>
       </c>
       <c r="AA44" s="12" t="n">
         <f aca="false">AA41*Допущения!$C$8</f>
-        <v>104694.907335022</v>
+        <v>74782.0766678727</v>
       </c>
       <c r="AB44" s="12" t="n">
         <f aca="false">AB41*Допущения!$C$8</f>
-        <v>83118.7795387093</v>
+        <v>59370.5568133638</v>
       </c>
       <c r="AC44" s="12" t="n">
         <f aca="false">AC41*Допущения!$C$8</f>
-        <v>87509.4866194674</v>
+        <v>62506.7761567624</v>
       </c>
       <c r="AD44" s="12" t="n">
         <f aca="false">AD41*Допущения!$C$8</f>
-        <v>152837.686469319</v>
+        <v>109169.776049514</v>
       </c>
       <c r="AE44" s="12" t="n">
         <f aca="false">AE41*Допущения!$C$8</f>
-        <v>175462.91859602</v>
+        <v>125330.656140014</v>
       </c>
       <c r="AF44" s="12" t="n">
         <f aca="false">AF41*Допущения!$C$8</f>
-        <v>199062.563148217</v>
+        <v>142187.545105869</v>
       </c>
       <c r="AG44" s="12" t="n">
         <f aca="false">AG41*Допущения!$C$8</f>
-        <v>223564.089803759</v>
+        <v>159688.635574114</v>
       </c>
       <c r="AH44" s="12" t="n">
         <f aca="false">AH41*Допущения!$C$8</f>
-        <v>142228.298733902</v>
+        <v>101591.641952787</v>
       </c>
       <c r="AI44" s="12" t="n">
         <f aca="false">AI41*Допущения!$C$8</f>
-        <v>165003.106692236</v>
+        <v>117859.361923025</v>
       </c>
       <c r="AJ44" s="12" t="n">
         <f aca="false">AJ41*Допущения!$C$8</f>
-        <v>188638.383478983</v>
+        <v>134741.702484988</v>
       </c>
       <c r="AK44" s="12" t="n">
         <f aca="false">AK41*Допущения!$C$8</f>
-        <v>193701.409822429</v>
+        <v>138358.149873164</v>
       </c>
       <c r="AL44" s="12" t="n">
         <f aca="false">AL41*Допущения!$C$8</f>
-        <v>198536.59998042</v>
+        <v>141811.857128871</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10385,147 +10385,147 @@
       </c>
       <c r="C45" s="33" t="n">
         <f aca="false">C41-C42-C43-C44</f>
-        <v>70150.16448</v>
+        <v>38974.0032</v>
       </c>
       <c r="D45" s="33" t="n">
         <f aca="false">D41-D42-D43-D44</f>
-        <v>102857.6786688</v>
+        <v>57145.632192</v>
       </c>
       <c r="E45" s="33" t="n">
         <f aca="false">E41-E42-E43-E44</f>
-        <v>150841.706488704</v>
+        <v>83804.58114336</v>
       </c>
       <c r="F45" s="33" t="n">
         <f aca="false">F41-F42-F43-F44</f>
-        <v>327777.421761187</v>
+        <v>182106.462319848</v>
       </c>
       <c r="G45" s="33" t="n">
         <f aca="false">G41-G42-G43-G44</f>
-        <v>440786.657720127</v>
+        <v>244892.093067</v>
       </c>
       <c r="H45" s="33" t="n">
         <f aca="false">H41-H42-H43-H44</f>
-        <v>564444.801035696</v>
+        <v>313594.039940711</v>
       </c>
       <c r="I45" s="33" t="n">
         <f aca="false">I41-I42-I43-I44</f>
-        <v>697959.201018181</v>
+        <v>387771.922355328</v>
       </c>
       <c r="J45" s="33" t="n">
         <f aca="false">J41-J42-J43-J44</f>
-        <v>480335.418001454</v>
+        <v>266864.579107285</v>
       </c>
       <c r="K45" s="33" t="n">
         <f aca="false">K41-K42-K43-K44</f>
-        <v>594979.299755312</v>
+        <v>330558.385778389</v>
       </c>
       <c r="L45" s="33" t="n">
         <f aca="false">L41-L42-L43-L44</f>
-        <v>719026.85145147</v>
+        <v>399476.680020402</v>
       </c>
       <c r="M45" s="33" t="n">
         <f aca="false">M41-M42-M43-M44</f>
-        <v>774358.348736154</v>
+        <v>430217.733419484</v>
       </c>
       <c r="N45" s="33" t="n">
         <f aca="false">N41-N42-N43-N44</f>
-        <v>827199.928643027</v>
+        <v>459575.439415607</v>
       </c>
       <c r="O45" s="33" t="n">
         <f aca="false">O41-O42-O43-O44</f>
-        <v>748897.686283273</v>
+        <v>416072.307713524</v>
       </c>
       <c r="P45" s="33" t="n">
         <f aca="false">P41-P42-P43-P44</f>
-        <v>624085.673400394</v>
+        <v>346729.294399811</v>
       </c>
       <c r="Q45" s="33" t="n">
         <f aca="false">Q41-Q42-Q43-Q44</f>
-        <v>683689.523697376</v>
+        <v>379843.98015182</v>
       </c>
       <c r="R45" s="33" t="n">
         <f aca="false">R41-R42-R43-R44</f>
-        <v>1234352.00121832</v>
+        <v>685780.841741647</v>
       </c>
       <c r="S45" s="33" t="n">
         <f aca="false">S41-S42-S43-S44</f>
-        <v>1457447.57087985</v>
+        <v>809728.1982496</v>
       </c>
       <c r="T45" s="33" t="n">
         <f aca="false">T41-T42-T43-T44</f>
-        <v>1693770.78958937</v>
+        <v>941024.56726731</v>
       </c>
       <c r="U45" s="33" t="n">
         <f aca="false">U41-U42-U43-U44</f>
-        <v>1942337.058196</v>
+        <v>1079122.92555197</v>
       </c>
       <c r="V45" s="33" t="n">
         <f aca="false">V41-V42-V43-V44</f>
-        <v>1258413.4888475</v>
+        <v>699148.914401313</v>
       </c>
       <c r="W45" s="33" t="n">
         <f aca="false">W41-W42-W43-W44</f>
-        <v>1483539.55048053</v>
+        <v>824224.37090991</v>
       </c>
       <c r="X45" s="33" t="n">
         <f aca="false">X41-X42-X43-X44</f>
-        <v>1720346.47678767</v>
+        <v>955789.478021071</v>
       </c>
       <c r="Y45" s="33" t="n">
         <f aca="false">Y41-Y42-Y43-Y44</f>
-        <v>1789077.06133223</v>
+        <v>993974.791510122</v>
       </c>
       <c r="Z45" s="33" t="n">
         <f aca="false">Z41-Z42-Z43-Z44</f>
-        <v>1854714.76957228</v>
+        <v>1030441.76589217</v>
       </c>
       <c r="AA45" s="33" t="n">
         <f aca="false">AA41-AA42-AA43-AA44</f>
-        <v>1580685.80107322</v>
+        <v>878196.849941616</v>
       </c>
       <c r="AB45" s="33" t="n">
         <f aca="false">AB41-AB42-AB43-AB44</f>
-        <v>1254928.99285869</v>
+        <v>697212.999370683</v>
       </c>
       <c r="AC45" s="33" t="n">
         <f aca="false">AC41-AC42-AC43-AC44</f>
-        <v>1321219.97602005</v>
+        <v>734042.919999002</v>
       </c>
       <c r="AD45" s="33" t="n">
         <f aca="false">AD41-AD42-AD43-AD44</f>
-        <v>2307546.44156525</v>
+        <v>1282025.82366508</v>
       </c>
       <c r="AE45" s="33" t="n">
         <f aca="false">AE41-AE42-AE43-AE44</f>
-        <v>2649142.6479043</v>
+        <v>1471809.72136016</v>
       </c>
       <c r="AF45" s="33" t="n">
         <f aca="false">AF41-AF42-AF43-AF44</f>
-        <v>3005450.55249666</v>
+        <v>1669767.13908977</v>
       </c>
       <c r="AG45" s="33" t="n">
         <f aca="false">AG41-AG42-AG43-AG44</f>
-        <v>3375375.0910905</v>
+        <v>1875289.68144996</v>
       </c>
       <c r="AH45" s="33" t="n">
         <f aca="false">AH41-AH42-AH43-AH44</f>
-        <v>2147365.69373011</v>
+        <v>1193032.6612829</v>
       </c>
       <c r="AI45" s="33" t="n">
         <f aca="false">AI41-AI42-AI43-AI44</f>
-        <v>2491220.19896129</v>
+        <v>1384071.22386581</v>
       </c>
       <c r="AJ45" s="33" t="n">
         <f aca="false">AJ41-AJ42-AJ43-AJ44</f>
-        <v>2848066.07974225</v>
+        <v>1582327.53021317</v>
       </c>
       <c r="AK45" s="33" t="n">
         <f aca="false">AK41-AK42-AK43-AK44</f>
-        <v>2924507.75255385</v>
+        <v>1624796.96735358</v>
       </c>
       <c r="AL45" s="33" t="n">
         <f aca="false">AL41-AL42-AL43-AL44</f>
-        <v>2997509.55008893</v>
+        <v>1665355.27982267</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11297,147 +11297,147 @@
       </c>
       <c r="C51" s="33" t="n">
         <f aca="false">C45-C50</f>
-        <v>-1279849.83552</v>
+        <v>-1311025.9968</v>
       </c>
       <c r="D51" s="33" t="n">
         <f aca="false">D45-D50</f>
-        <v>-447142.3213312</v>
+        <v>-492854.367808</v>
       </c>
       <c r="E51" s="33" t="n">
         <f aca="false">E45-E50</f>
-        <v>-399158.293511296</v>
+        <v>-466195.41885664</v>
       </c>
       <c r="F51" s="33" t="n">
         <f aca="false">F45-F50</f>
-        <v>-222222.578238813</v>
+        <v>-367893.537680152</v>
       </c>
       <c r="G51" s="33" t="n">
         <f aca="false">G45-G50</f>
-        <v>-109213.342279873</v>
+        <v>-305107.906933</v>
       </c>
       <c r="H51" s="33" t="n">
         <f aca="false">H45-H50</f>
-        <v>14444.8010356961</v>
+        <v>-236405.960059289</v>
       </c>
       <c r="I51" s="33" t="n">
         <f aca="false">I45-I50</f>
-        <v>147959.201018181</v>
+        <v>-162228.077644672</v>
       </c>
       <c r="J51" s="33" t="n">
         <f aca="false">J45-J50</f>
-        <v>-69664.5819985462</v>
+        <v>-283135.420892715</v>
       </c>
       <c r="K51" s="33" t="n">
         <f aca="false">K45-K50</f>
-        <v>44979.2997553118</v>
+        <v>-219441.614221611</v>
       </c>
       <c r="L51" s="33" t="n">
         <f aca="false">L45-L50</f>
-        <v>169026.85145147</v>
+        <v>-150523.319979598</v>
       </c>
       <c r="M51" s="33" t="n">
         <f aca="false">M45-M50</f>
-        <v>224358.348736154</v>
+        <v>-119782.266580516</v>
       </c>
       <c r="N51" s="33" t="n">
         <f aca="false">N45-N50</f>
-        <v>277199.928643027</v>
+        <v>-90424.5605843931</v>
       </c>
       <c r="O51" s="33" t="n">
         <f aca="false">O45-O50</f>
-        <v>-461102.313716728</v>
+        <v>-793927.692286476</v>
       </c>
       <c r="P51" s="33" t="n">
         <f aca="false">P45-P50</f>
-        <v>-585914.326599606</v>
+        <v>-863270.705600189</v>
       </c>
       <c r="Q51" s="33" t="n">
         <f aca="false">Q45-Q50</f>
-        <v>-526310.476302624</v>
+        <v>-830156.01984818</v>
       </c>
       <c r="R51" s="33" t="n">
         <f aca="false">R45-R50</f>
-        <v>24352.0012183241</v>
+        <v>-524219.158258353</v>
       </c>
       <c r="S51" s="33" t="n">
         <f aca="false">S45-S50</f>
-        <v>247447.570879849</v>
+        <v>-400271.8017504</v>
       </c>
       <c r="T51" s="33" t="n">
         <f aca="false">T45-T50</f>
-        <v>483770.78958937</v>
+        <v>-268975.43273269</v>
       </c>
       <c r="U51" s="33" t="n">
         <f aca="false">U45-U50</f>
-        <v>732337.058196003</v>
+        <v>-130877.074448029</v>
       </c>
       <c r="V51" s="33" t="n">
         <f aca="false">V45-V50</f>
-        <v>48413.4888474974</v>
+        <v>-510851.085598687</v>
       </c>
       <c r="W51" s="33" t="n">
         <f aca="false">W45-W50</f>
-        <v>273539.550480529</v>
+        <v>-385775.62909009</v>
       </c>
       <c r="X51" s="33" t="n">
         <f aca="false">X45-X50</f>
-        <v>510346.476787673</v>
+        <v>-254210.521978929</v>
       </c>
       <c r="Y51" s="33" t="n">
         <f aca="false">Y45-Y50</f>
-        <v>579077.061332228</v>
+        <v>-216025.208489878</v>
       </c>
       <c r="Z51" s="33" t="n">
         <f aca="false">Z45-Z50</f>
-        <v>644714.769572278</v>
+        <v>-179558.234107832</v>
       </c>
       <c r="AA51" s="33" t="n">
         <f aca="false">AA45-AA50</f>
-        <v>-209314.19892678</v>
+        <v>-911803.150058384</v>
       </c>
       <c r="AB51" s="33" t="n">
         <f aca="false">AB45-AB50</f>
-        <v>-535071.007141306</v>
+        <v>-1092787.00062932</v>
       </c>
       <c r="AC51" s="33" t="n">
         <f aca="false">AC45-AC50</f>
-        <v>-468780.023979948</v>
+        <v>-1055957.080001</v>
       </c>
       <c r="AD51" s="33" t="n">
         <f aca="false">AD45-AD50</f>
-        <v>517546.441565251</v>
+        <v>-507974.176334922</v>
       </c>
       <c r="AE51" s="33" t="n">
         <f aca="false">AE45-AE50</f>
-        <v>859142.647904296</v>
+        <v>-318190.278639836</v>
       </c>
       <c r="AF51" s="33" t="n">
         <f aca="false">AF45-AF50</f>
-        <v>1215450.55249666</v>
+        <v>-120232.860910229</v>
       </c>
       <c r="AG51" s="33" t="n">
         <f aca="false">AG45-AG50</f>
-        <v>1585375.0910905</v>
+        <v>85289.6814499588</v>
       </c>
       <c r="AH51" s="33" t="n">
         <f aca="false">AH45-AH50</f>
-        <v>357365.693730108</v>
+        <v>-596967.338717101</v>
       </c>
       <c r="AI51" s="33" t="n">
         <f aca="false">AI45-AI50</f>
-        <v>701220.198961286</v>
+        <v>-405928.776134186</v>
       </c>
       <c r="AJ51" s="33" t="n">
         <f aca="false">AJ45-AJ50</f>
-        <v>1058066.07974225</v>
+        <v>-207672.46978683</v>
       </c>
       <c r="AK51" s="33" t="n">
         <f aca="false">AK45-AK50</f>
-        <v>1134507.75255385</v>
+        <v>-165203.032646423</v>
       </c>
       <c r="AL51" s="33" t="n">
         <f aca="false">AL45-AL50</f>
-        <v>1207509.55008893</v>
+        <v>-124644.720177334</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11449,147 +11449,147 @@
       </c>
       <c r="C52" s="33" t="n">
         <f aca="false">C51</f>
-        <v>-1279849.83552</v>
+        <v>-1311025.9968</v>
       </c>
       <c r="D52" s="33" t="n">
         <f aca="false">C52+D51</f>
-        <v>-1726992.1568512</v>
+        <v>-1803880.364608</v>
       </c>
       <c r="E52" s="33" t="n">
         <f aca="false">D52+E51</f>
-        <v>-2126150.4503625</v>
+        <v>-2270075.78346464</v>
       </c>
       <c r="F52" s="33" t="n">
         <f aca="false">E52+F51</f>
-        <v>-2348373.02860131</v>
+        <v>-2637969.32114479</v>
       </c>
       <c r="G52" s="33" t="n">
         <f aca="false">F52+G51</f>
-        <v>-2457586.37088118</v>
+        <v>-2943077.22807779</v>
       </c>
       <c r="H52" s="33" t="n">
         <f aca="false">G52+H51</f>
-        <v>-2443141.56984549</v>
+        <v>-3179483.18813708</v>
       </c>
       <c r="I52" s="33" t="n">
         <f aca="false">H52+I51</f>
-        <v>-2295182.36882731</v>
+        <v>-3341711.26578175</v>
       </c>
       <c r="J52" s="33" t="n">
         <f aca="false">I52+J51</f>
-        <v>-2364846.95082585</v>
+        <v>-3624846.68667447</v>
       </c>
       <c r="K52" s="33" t="n">
         <f aca="false">J52+K51</f>
-        <v>-2319867.65107054</v>
+        <v>-3844288.30089608</v>
       </c>
       <c r="L52" s="33" t="n">
         <f aca="false">K52+L51</f>
-        <v>-2150840.79961907</v>
+        <v>-3994811.62087568</v>
       </c>
       <c r="M52" s="33" t="n">
         <f aca="false">L52+M51</f>
-        <v>-1926482.45088292</v>
+        <v>-4114593.88745619</v>
       </c>
       <c r="N52" s="33" t="n">
         <f aca="false">M52+N51</f>
-        <v>-1649282.52223989</v>
+        <v>-4205018.44804059</v>
       </c>
       <c r="O52" s="33" t="n">
         <f aca="false">N52+O51</f>
-        <v>-2110384.83595662</v>
+        <v>-4998946.14032706</v>
       </c>
       <c r="P52" s="33" t="n">
         <f aca="false">O52+P51</f>
-        <v>-2696299.16255622</v>
+        <v>-5862216.84592725</v>
       </c>
       <c r="Q52" s="33" t="n">
         <f aca="false">P52+Q51</f>
-        <v>-3222609.63885885</v>
+        <v>-6692372.86577543</v>
       </c>
       <c r="R52" s="33" t="n">
         <f aca="false">Q52+R51</f>
-        <v>-3198257.63764052</v>
+        <v>-7216592.02403379</v>
       </c>
       <c r="S52" s="33" t="n">
         <f aca="false">R52+S51</f>
-        <v>-2950810.06676067</v>
+        <v>-7616863.82578419</v>
       </c>
       <c r="T52" s="33" t="n">
         <f aca="false">S52+T51</f>
-        <v>-2467039.2771713</v>
+        <v>-7885839.25851687</v>
       </c>
       <c r="U52" s="33" t="n">
         <f aca="false">T52+U51</f>
-        <v>-1734702.2189753</v>
+        <v>-8016716.3329649</v>
       </c>
       <c r="V52" s="33" t="n">
         <f aca="false">U52+V51</f>
-        <v>-1686288.7301278</v>
+        <v>-8527567.41856359</v>
       </c>
       <c r="W52" s="33" t="n">
         <f aca="false">V52+W51</f>
-        <v>-1412749.17964727</v>
+        <v>-8913343.04765368</v>
       </c>
       <c r="X52" s="33" t="n">
         <f aca="false">W52+X51</f>
-        <v>-902402.7028596</v>
+        <v>-9167553.56963261</v>
       </c>
       <c r="Y52" s="33" t="n">
         <f aca="false">X52+Y51</f>
-        <v>-323325.641527373</v>
+        <v>-9383578.77812249</v>
       </c>
       <c r="Z52" s="33" t="n">
         <f aca="false">Y52+Z51</f>
-        <v>321389.128044906</v>
+        <v>-9563137.01223032</v>
       </c>
       <c r="AA52" s="33" t="n">
         <f aca="false">Z52+AA51</f>
-        <v>112074.929118125</v>
+        <v>-10474940.1622887</v>
       </c>
       <c r="AB52" s="33" t="n">
         <f aca="false">AA52+AB51</f>
-        <v>-422996.078023181</v>
+        <v>-11567727.162918</v>
       </c>
       <c r="AC52" s="33" t="n">
         <f aca="false">AB52+AC51</f>
-        <v>-891776.102003129</v>
+        <v>-12623684.242919</v>
       </c>
       <c r="AD52" s="33" t="n">
         <f aca="false">AC52+AD51</f>
-        <v>-374229.660437878</v>
+        <v>-13131658.4192539</v>
       </c>
       <c r="AE52" s="33" t="n">
         <f aca="false">AD52+AE51</f>
-        <v>484912.987466418</v>
+        <v>-13449848.6978938</v>
       </c>
       <c r="AF52" s="33" t="n">
         <f aca="false">AE52+AF51</f>
-        <v>1700363.53996308</v>
+        <v>-13570081.558804</v>
       </c>
       <c r="AG52" s="33" t="n">
         <f aca="false">AF52+AG51</f>
-        <v>3285738.63105357</v>
+        <v>-13484791.877354</v>
       </c>
       <c r="AH52" s="33" t="n">
         <f aca="false">AG52+AH51</f>
-        <v>3643104.32478368</v>
+        <v>-14081759.2160711</v>
       </c>
       <c r="AI52" s="33" t="n">
         <f aca="false">AH52+AI51</f>
-        <v>4344324.52374497</v>
+        <v>-14487687.9922053</v>
       </c>
       <c r="AJ52" s="33" t="n">
         <f aca="false">AI52+AJ51</f>
-        <v>5402390.60348722</v>
+        <v>-14695360.4619922</v>
       </c>
       <c r="AK52" s="33" t="n">
         <f aca="false">AJ52+AK51</f>
-        <v>6536898.35604107</v>
+        <v>-14860563.4946386</v>
       </c>
       <c r="AL52" s="33" t="n">
         <f aca="false">AK52+AL51</f>
-        <v>7744407.90613</v>
+        <v>-14985208.2148159</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11617,33 +11617,33 @@
         <f aca="false">IF(G51&gt;0,G$4,"")</f>
         <v/>
       </c>
-      <c r="H53" s="34" t="n">
+      <c r="H53" s="34" t="str">
         <f aca="false">IF(H51&gt;0,H$4,"")</f>
-        <v>6</v>
-      </c>
-      <c r="I53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="I53" s="34" t="str">
         <f aca="false">IF(I51&gt;0,I$4,"")</f>
-        <v>7</v>
+        <v/>
       </c>
       <c r="J53" s="34" t="str">
         <f aca="false">IF(J51&gt;0,J$4,"")</f>
         <v/>
       </c>
-      <c r="K53" s="34" t="n">
+      <c r="K53" s="34" t="str">
         <f aca="false">IF(K51&gt;0,K$4,"")</f>
-        <v>9</v>
-      </c>
-      <c r="L53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="L53" s="34" t="str">
         <f aca="false">IF(L51&gt;0,L$4,"")</f>
-        <v>10</v>
-      </c>
-      <c r="M53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="M53" s="34" t="str">
         <f aca="false">IF(M51&gt;0,M$4,"")</f>
-        <v>11</v>
-      </c>
-      <c r="N53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="N53" s="34" t="str">
         <f aca="false">IF(N51&gt;0,N$4,"")</f>
-        <v>12</v>
+        <v/>
       </c>
       <c r="O53" s="34" t="str">
         <f aca="false">IF(O51&gt;0,O$4,"")</f>
@@ -11657,41 +11657,41 @@
         <f aca="false">IF(Q51&gt;0,Q$4,"")</f>
         <v/>
       </c>
-      <c r="R53" s="34" t="n">
+      <c r="R53" s="34" t="str">
         <f aca="false">IF(R51&gt;0,R$4,"")</f>
-        <v>16</v>
-      </c>
-      <c r="S53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="S53" s="34" t="str">
         <f aca="false">IF(S51&gt;0,S$4,"")</f>
-        <v>17</v>
-      </c>
-      <c r="T53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="T53" s="34" t="str">
         <f aca="false">IF(T51&gt;0,T$4,"")</f>
-        <v>18</v>
-      </c>
-      <c r="U53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="U53" s="34" t="str">
         <f aca="false">IF(U51&gt;0,U$4,"")</f>
-        <v>19</v>
-      </c>
-      <c r="V53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="V53" s="34" t="str">
         <f aca="false">IF(V51&gt;0,V$4,"")</f>
-        <v>20</v>
-      </c>
-      <c r="W53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="W53" s="34" t="str">
         <f aca="false">IF(W51&gt;0,W$4,"")</f>
-        <v>21</v>
-      </c>
-      <c r="X53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="X53" s="34" t="str">
         <f aca="false">IF(X51&gt;0,X$4,"")</f>
-        <v>22</v>
-      </c>
-      <c r="Y53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="Y53" s="34" t="str">
         <f aca="false">IF(Y51&gt;0,Y$4,"")</f>
-        <v>23</v>
-      </c>
-      <c r="Z53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="Z53" s="34" t="str">
         <f aca="false">IF(Z51&gt;0,Z$4,"")</f>
-        <v>24</v>
+        <v/>
       </c>
       <c r="AA53" s="34" t="str">
         <f aca="false">IF(AA51&gt;0,AA$4,"")</f>
@@ -11705,41 +11705,41 @@
         <f aca="false">IF(AC51&gt;0,AC$4,"")</f>
         <v/>
       </c>
-      <c r="AD53" s="34" t="n">
+      <c r="AD53" s="34" t="str">
         <f aca="false">IF(AD51&gt;0,AD$4,"")</f>
-        <v>28</v>
-      </c>
-      <c r="AE53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AE53" s="34" t="str">
         <f aca="false">IF(AE51&gt;0,AE$4,"")</f>
-        <v>29</v>
-      </c>
-      <c r="AF53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AF53" s="34" t="str">
         <f aca="false">IF(AF51&gt;0,AF$4,"")</f>
-        <v>30</v>
+        <v/>
       </c>
       <c r="AG53" s="34" t="n">
         <f aca="false">IF(AG51&gt;0,AG$4,"")</f>
         <v>31</v>
       </c>
-      <c r="AH53" s="34" t="n">
+      <c r="AH53" s="34" t="str">
         <f aca="false">IF(AH51&gt;0,AH$4,"")</f>
-        <v>32</v>
-      </c>
-      <c r="AI53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AI53" s="34" t="str">
         <f aca="false">IF(AI51&gt;0,AI$4,"")</f>
-        <v>33</v>
-      </c>
-      <c r="AJ53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AJ53" s="34" t="str">
         <f aca="false">IF(AJ51&gt;0,AJ$4,"")</f>
-        <v>34</v>
-      </c>
-      <c r="AK53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AK53" s="34" t="str">
         <f aca="false">IF(AK51&gt;0,AK$4,"")</f>
-        <v>35</v>
-      </c>
-      <c r="AL53" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AL53" s="34" t="str">
         <f aca="false">IF(AL51&gt;0,AL$4,"")</f>
-        <v>36</v>
+        <v/>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11839,13 +11839,13 @@
         <f aca="false">IF(Y52&gt;=0,Y$4,"")</f>
         <v/>
       </c>
-      <c r="Z54" s="34" t="n">
+      <c r="Z54" s="34" t="str">
         <f aca="false">IF(Z52&gt;=0,Z$4,"")</f>
-        <v>24</v>
-      </c>
-      <c r="AA54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AA54" s="34" t="str">
         <f aca="false">IF(AA52&gt;=0,AA$4,"")</f>
-        <v>25</v>
+        <v/>
       </c>
       <c r="AB54" s="34" t="str">
         <f aca="false">IF(AB52&gt;=0,AB$4,"")</f>
@@ -11859,37 +11859,37 @@
         <f aca="false">IF(AD52&gt;=0,AD$4,"")</f>
         <v/>
       </c>
-      <c r="AE54" s="34" t="n">
+      <c r="AE54" s="34" t="str">
         <f aca="false">IF(AE52&gt;=0,AE$4,"")</f>
-        <v>29</v>
-      </c>
-      <c r="AF54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AF54" s="34" t="str">
         <f aca="false">IF(AF52&gt;=0,AF$4,"")</f>
-        <v>30</v>
-      </c>
-      <c r="AG54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AG54" s="34" t="str">
         <f aca="false">IF(AG52&gt;=0,AG$4,"")</f>
-        <v>31</v>
-      </c>
-      <c r="AH54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AH54" s="34" t="str">
         <f aca="false">IF(AH52&gt;=0,AH$4,"")</f>
-        <v>32</v>
-      </c>
-      <c r="AI54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AI54" s="34" t="str">
         <f aca="false">IF(AI52&gt;=0,AI$4,"")</f>
-        <v>33</v>
-      </c>
-      <c r="AJ54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AJ54" s="34" t="str">
         <f aca="false">IF(AJ52&gt;=0,AJ$4,"")</f>
-        <v>34</v>
-      </c>
-      <c r="AK54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AK54" s="34" t="str">
         <f aca="false">IF(AK52&gt;=0,AK$4,"")</f>
-        <v>35</v>
-      </c>
-      <c r="AL54" s="34" t="n">
+        <v/>
+      </c>
+      <c r="AL54" s="34" t="str">
         <f aca="false">IF(AL52&gt;=0,AL$4,"")</f>
-        <v>36</v>
+        <v/>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13087,147 +13087,147 @@
       </c>
       <c r="C65" s="12" t="n">
         <f aca="false">C64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>384993</v>
+        <v>274995</v>
       </c>
       <c r="D65" s="12" t="n">
         <f aca="false">D64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>567383.43375</v>
+        <v>405273.88125</v>
       </c>
       <c r="E65" s="12" t="n">
         <f aca="false">E64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>836269.76356875</v>
+        <v>597335.54540625</v>
       </c>
       <c r="F65" s="12" t="n">
         <f aca="false">F64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>1826241.78640641</v>
+        <v>1304458.41886172</v>
       </c>
       <c r="G65" s="12" t="n">
         <f aca="false">G64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2467921.0312704</v>
+        <v>1762800.73662172</v>
       </c>
       <c r="H65" s="12" t="n">
         <f aca="false">H64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3175537.27655557</v>
+        <v>2268240.91182541</v>
       </c>
       <c r="I65" s="12" t="n">
         <f aca="false">I64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3945373.21953247</v>
+        <v>2818123.72823748</v>
       </c>
       <c r="J65" s="12" t="n">
         <f aca="false">J64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>2727937.71190697</v>
+        <v>1948526.93707641</v>
       </c>
       <c r="K65" s="12" t="n">
         <f aca="false">K64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3394634.50348901</v>
+        <v>2424738.93106358</v>
       </c>
       <c r="L65" s="12" t="n">
         <f aca="false">L64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4121043.80096321</v>
+        <v>2943602.71497372</v>
       </c>
       <c r="M65" s="12" t="n">
         <f aca="false">M64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4458048.5179295</v>
+        <v>3184320.36994964</v>
       </c>
       <c r="N65" s="12" t="n">
         <f aca="false">N64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4783258.06980197</v>
+        <v>3416612.90700141</v>
       </c>
       <c r="O65" s="12" t="n">
         <f aca="false">O64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>4308664.02988712</v>
+        <v>3077617.16420509</v>
       </c>
       <c r="P65" s="12" t="n">
         <f aca="false">P64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3580387.1916308</v>
+        <v>2557419.42259343</v>
       </c>
       <c r="Q65" s="12" t="n">
         <f aca="false">Q64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>3917065.23992372</v>
+        <v>2797903.74280266</v>
       </c>
       <c r="R65" s="12" t="n">
         <f aca="false">R64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>7069932.59421066</v>
+        <v>5049951.85300761</v>
       </c>
       <c r="S65" s="12" t="n">
         <f aca="false">S64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>8351718.04875461</v>
+        <v>5965512.89196758</v>
       </c>
       <c r="T65" s="12" t="n">
         <f aca="false">T64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>9716064.56405258</v>
+        <v>6940046.11718042</v>
       </c>
       <c r="U65" s="12" t="n">
         <f aca="false">U64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>11158317.62967</v>
+        <v>7970226.87833569</v>
       </c>
       <c r="V65" s="12" t="n">
         <f aca="false">V64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>7242312.80777325</v>
+        <v>5173080.57698089</v>
       </c>
       <c r="W65" s="12" t="n">
         <f aca="false">W64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>8555423.24193883</v>
+        <v>6111016.60138488</v>
       </c>
       <c r="X65" s="12" t="n">
         <f aca="false">X64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>9943300.9205233</v>
+        <v>7102357.80037379</v>
       </c>
       <c r="Y65" s="12" t="n">
         <f aca="false">Y64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>10365271.388305</v>
+        <v>7403765.2773607</v>
       </c>
       <c r="Z65" s="12" t="n">
         <f aca="false">Z64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>10772472.8897143</v>
+        <v>7694623.49265308</v>
       </c>
       <c r="AA65" s="12" t="n">
         <f aca="false">AA64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>9163333.67085945</v>
+        <v>6545238.33632818</v>
       </c>
       <c r="AB65" s="12" t="n">
         <f aca="false">AB64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>7267201.19428452</v>
+        <v>5190857.99591752</v>
       </c>
       <c r="AC65" s="12" t="n">
         <f aca="false">AC64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>7648087.60248457</v>
+        <v>5462919.71606041</v>
       </c>
       <c r="AD65" s="12" t="n">
         <f aca="false">AD64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>13359404.9773293</v>
+        <v>9542432.12666382</v>
       </c>
       <c r="AE65" s="12" t="n">
         <f aca="false">AE64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>15345612.2084351</v>
+        <v>10961151.5774536</v>
       </c>
       <c r="AF65" s="12" t="n">
         <f aca="false">AF64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>17425221.3885162</v>
+        <v>12446586.706083</v>
       </c>
       <c r="AG65" s="12" t="n">
         <f aca="false">AG64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>19592966.8349113</v>
+        <v>13994976.310651</v>
       </c>
       <c r="AH65" s="12" t="n">
         <f aca="false">AH64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>12482192.5973473</v>
+        <v>8915851.8552481</v>
       </c>
       <c r="AI65" s="12" t="n">
         <f aca="false">AI64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>14503838.0134952</v>
+        <v>10359884.2953537</v>
       </c>
       <c r="AJ65" s="12" t="n">
         <f aca="false">AJ64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>16610068.175581</v>
+        <v>11864334.4111293</v>
       </c>
       <c r="AK65" s="12" t="n">
         <f aca="false">AK64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>17087446.5394356</v>
+        <v>12205318.9567397</v>
       </c>
       <c r="AL65" s="12" t="n">
         <f aca="false">AL64*(Допущения!$C$6+Допущения!$C$7)*(1-Допущения!$C$13)</f>
-        <v>17548116.6605554</v>
+        <v>12534369.0432539</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13239,147 +13239,147 @@
       </c>
       <c r="C66" s="12" t="n">
         <f aca="false">C64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>91003.5</v>
+        <v>89302.5</v>
       </c>
       <c r="D66" s="12" t="n">
         <f aca="false">D64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>134116.408125</v>
+        <v>131609.559375</v>
       </c>
       <c r="E66" s="12" t="n">
         <f aca="false">E64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>197674.958840625</v>
+        <v>193980.099796875</v>
       </c>
       <c r="F66" s="12" t="n">
         <f aca="false">F64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>431681.600468672</v>
+        <v>423612.785506641</v>
       </c>
       <c r="G66" s="12" t="n">
         <f aca="false">G64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>583359.831397495</v>
+        <v>572455.909315299</v>
       </c>
       <c r="H66" s="12" t="n">
         <f aca="false">H64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>750624.054325727</v>
+        <v>736593.698170106</v>
       </c>
       <c r="I66" s="12" t="n">
         <f aca="false">I64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>932595.584293021</v>
+        <v>915163.891128665</v>
       </c>
       <c r="J66" s="12" t="n">
         <f aca="false">J64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>644821.800826317</v>
+        <v>632769.056885638</v>
       </c>
       <c r="K66" s="12" t="n">
         <f aca="false">K64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>802413.60502207</v>
+        <v>787415.219881471</v>
       </c>
       <c r="L66" s="12" t="n">
         <f aca="false">L64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>974120.073718109</v>
+        <v>955912.22187291</v>
       </c>
       <c r="M66" s="12" t="n">
         <f aca="false">M64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1053780.24613797</v>
+        <v>1034083.41910736</v>
       </c>
       <c r="N66" s="12" t="n">
         <f aca="false">N64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1130652.31252315</v>
+        <v>1109518.6244386</v>
       </c>
       <c r="O66" s="12" t="n">
         <f aca="false">O64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1018469.18526787</v>
+        <v>999432.3780666</v>
       </c>
       <c r="P66" s="12" t="n">
         <f aca="false">P64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>846321.27283762</v>
+        <v>830502.183625702</v>
       </c>
       <c r="Q66" s="12" t="n">
         <f aca="false">Q64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>925904.228288303</v>
+        <v>908597.607198802</v>
       </c>
       <c r="R66" s="12" t="n">
         <f aca="false">R64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1671169.63383035</v>
+        <v>1639932.81824474</v>
       </c>
       <c r="S66" s="12" t="n">
         <f aca="false">S64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1974154.26631092</v>
+        <v>1937254.18656679</v>
       </c>
       <c r="T66" s="12" t="n">
         <f aca="false">T64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2296654.43671641</v>
+        <v>2253726.31640395</v>
       </c>
       <c r="U66" s="12" t="n">
         <f aca="false">U64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2637569.92571728</v>
+        <v>2588269.55327396</v>
       </c>
       <c r="V66" s="12" t="n">
         <f aca="false">V64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1711916.35588749</v>
+        <v>1679917.91932885</v>
       </c>
       <c r="W66" s="12" t="n">
         <f aca="false">W64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2022305.49386036</v>
+        <v>1984505.39117138</v>
       </c>
       <c r="X66" s="12" t="n">
         <f aca="false">X64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2350367.89063916</v>
+        <v>2306435.78053376</v>
       </c>
       <c r="Y66" s="12" t="n">
         <f aca="false">Y64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2450112.01446679</v>
+        <v>2404315.52821507</v>
       </c>
       <c r="Z66" s="12" t="n">
         <f aca="false">Z64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2546365.09396045</v>
+        <v>2498769.48472755</v>
       </c>
       <c r="AA66" s="12" t="n">
         <f aca="false">AA64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2166001.55253747</v>
+        <v>2125515.54220967</v>
       </c>
       <c r="AB66" s="12" t="n">
         <f aca="false">AB64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1717799.39864899</v>
+        <v>1685690.99867425</v>
       </c>
       <c r="AC66" s="12" t="n">
         <f aca="false">AC64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>1807832.19469628</v>
+        <v>1774040.93872065</v>
       </c>
       <c r="AD66" s="12" t="n">
         <f aca="false">AD64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>3157856.40480318</v>
+        <v>3098831.05144237</v>
       </c>
       <c r="AE66" s="12" t="n">
         <f aca="false">AE64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>3627350.16119858</v>
+        <v>3559549.22360608</v>
       </c>
       <c r="AF66" s="12" t="n">
         <f aca="false">AF64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>4118921.99242541</v>
+        <v>4041932.79630531</v>
       </c>
       <c r="AG66" s="12" t="n">
         <f aca="false">AG64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>4631327.2120814</v>
+        <v>4544760.34830418</v>
       </c>
       <c r="AH66" s="12" t="n">
         <f aca="false">AH64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>2950503.55209757</v>
+        <v>2895353.95299294</v>
       </c>
       <c r="AI66" s="12" t="n">
         <f aca="false">AI64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>3428374.08124592</v>
+        <v>3364292.32271796</v>
       </c>
       <c r="AJ66" s="12" t="n">
         <f aca="false">AJ64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>3926238.50100257</v>
+        <v>3852850.86546981</v>
       </c>
       <c r="AK66" s="12" t="n">
         <f aca="false">AK64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>4039079.77846748</v>
+        <v>3963582.96017837</v>
       </c>
       <c r="AL66" s="12" t="n">
         <f aca="false">AL64*(1+Допущения!$C$6)*Допущения!$E$23</f>
-        <v>4147971.61122112</v>
+        <v>4070439.43157213</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13543,147 +13543,147 @@
       </c>
       <c r="C68" s="12" t="n">
         <f aca="false">C65*Допущения!$C$8</f>
-        <v>15399.72</v>
+        <v>10999.8</v>
       </c>
       <c r="D68" s="12" t="n">
         <f aca="false">D65*Допущения!$C$8</f>
-        <v>22695.33735</v>
+        <v>16210.95525</v>
       </c>
       <c r="E68" s="12" t="n">
         <f aca="false">E65*Допущения!$C$8</f>
-        <v>33450.79054275</v>
+        <v>23893.42181625</v>
       </c>
       <c r="F68" s="12" t="n">
         <f aca="false">F65*Допущения!$C$8</f>
-        <v>73049.6714562563</v>
+        <v>52178.3367544687</v>
       </c>
       <c r="G68" s="12" t="n">
         <f aca="false">G65*Допущения!$C$8</f>
-        <v>98716.841250816</v>
+        <v>70512.0294648686</v>
       </c>
       <c r="H68" s="12" t="n">
         <f aca="false">H65*Допущения!$C$8</f>
-        <v>127021.491062223</v>
+        <v>90729.6364730162</v>
       </c>
       <c r="I68" s="12" t="n">
         <f aca="false">I65*Допущения!$C$8</f>
-        <v>157814.928781299</v>
+        <v>112724.949129499</v>
       </c>
       <c r="J68" s="12" t="n">
         <f aca="false">J65*Допущения!$C$8</f>
-        <v>109117.508476279</v>
+        <v>77941.0774830564</v>
       </c>
       <c r="K68" s="12" t="n">
         <f aca="false">K65*Допущения!$C$8</f>
-        <v>135785.38013956</v>
+        <v>96989.557242543</v>
       </c>
       <c r="L68" s="12" t="n">
         <f aca="false">L65*Допущения!$C$8</f>
-        <v>164841.752038529</v>
+        <v>117744.108598949</v>
       </c>
       <c r="M68" s="12" t="n">
         <f aca="false">M65*Допущения!$C$8</f>
-        <v>178321.94071718</v>
+        <v>127372.814797986</v>
       </c>
       <c r="N68" s="12" t="n">
         <f aca="false">N65*Допущения!$C$8</f>
-        <v>191330.322792079</v>
+        <v>136664.516280056</v>
       </c>
       <c r="O68" s="12" t="n">
         <f aca="false">O65*Допущения!$C$8</f>
-        <v>172346.561195485</v>
+        <v>123104.686568203</v>
       </c>
       <c r="P68" s="12" t="n">
         <f aca="false">P65*Допущения!$C$8</f>
-        <v>143215.487665232</v>
+        <v>102296.776903737</v>
       </c>
       <c r="Q68" s="12" t="n">
         <f aca="false">Q65*Допущения!$C$8</f>
-        <v>156682.609596949</v>
+        <v>111916.149712106</v>
       </c>
       <c r="R68" s="12" t="n">
         <f aca="false">R65*Допущения!$C$8</f>
-        <v>282797.303768426</v>
+        <v>201998.074120304</v>
       </c>
       <c r="S68" s="12" t="n">
         <f aca="false">S65*Допущения!$C$8</f>
-        <v>334068.721950185</v>
+        <v>238620.515678703</v>
       </c>
       <c r="T68" s="12" t="n">
         <f aca="false">T65*Допущения!$C$8</f>
-        <v>388642.582562103</v>
+        <v>277601.844687217</v>
       </c>
       <c r="U68" s="12" t="n">
         <f aca="false">U65*Допущения!$C$8</f>
-        <v>446332.705186799</v>
+        <v>318809.075133428</v>
       </c>
       <c r="V68" s="12" t="n">
         <f aca="false">V65*Допущения!$C$8</f>
-        <v>289692.51231093</v>
+        <v>206923.223079236</v>
       </c>
       <c r="W68" s="12" t="n">
         <f aca="false">W65*Допущения!$C$8</f>
-        <v>342216.929677553</v>
+        <v>244440.664055395</v>
       </c>
       <c r="X68" s="12" t="n">
         <f aca="false">X65*Допущения!$C$8</f>
-        <v>397732.036820932</v>
+        <v>284094.312014951</v>
       </c>
       <c r="Y68" s="12" t="n">
         <f aca="false">Y65*Допущения!$C$8</f>
-        <v>414610.855532199</v>
+        <v>296150.611094428</v>
       </c>
       <c r="Z68" s="12" t="n">
         <f aca="false">Z65*Допущения!$C$8</f>
-        <v>430898.915588572</v>
+        <v>307784.939706123</v>
       </c>
       <c r="AA68" s="12" t="n">
         <f aca="false">AA65*Допущения!$C$8</f>
-        <v>366533.346834378</v>
+        <v>261809.533453127</v>
       </c>
       <c r="AB68" s="12" t="n">
         <f aca="false">AB65*Допущения!$C$8</f>
-        <v>290688.047771381</v>
+        <v>207634.319836701</v>
       </c>
       <c r="AC68" s="12" t="n">
         <f aca="false">AC65*Допущения!$C$8</f>
-        <v>305923.504099383</v>
+        <v>218516.788642416</v>
       </c>
       <c r="AD68" s="12" t="n">
         <f aca="false">AD65*Допущения!$C$8</f>
-        <v>534376.199093174</v>
+        <v>381697.285066553</v>
       </c>
       <c r="AE68" s="12" t="n">
         <f aca="false">AE65*Допущения!$C$8</f>
-        <v>613824.488337404</v>
+        <v>438446.063098146</v>
       </c>
       <c r="AF68" s="12" t="n">
         <f aca="false">AF65*Допущения!$C$8</f>
-        <v>697008.855540649</v>
+        <v>497863.468243321</v>
       </c>
       <c r="AG68" s="12" t="n">
         <f aca="false">AG65*Допущения!$C$8</f>
-        <v>783718.673396454</v>
+        <v>559799.052426038</v>
       </c>
       <c r="AH68" s="12" t="n">
         <f aca="false">AH65*Допущения!$C$8</f>
-        <v>499287.703893894</v>
+        <v>356634.074209924</v>
       </c>
       <c r="AI68" s="12" t="n">
         <f aca="false">AI65*Допущения!$C$8</f>
-        <v>580153.520539809</v>
+        <v>414395.371814149</v>
       </c>
       <c r="AJ68" s="12" t="n">
         <f aca="false">AJ65*Допущения!$C$8</f>
-        <v>664402.727023239</v>
+        <v>474573.376445171</v>
       </c>
       <c r="AK68" s="12" t="n">
         <f aca="false">AK65*Допущения!$C$8</f>
-        <v>683497.861577426</v>
+        <v>488212.75826959</v>
       </c>
       <c r="AL68" s="12" t="n">
         <f aca="false">AL65*Допущения!$C$8</f>
-        <v>701924.666422216</v>
+        <v>501374.761730154</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13695,147 +13695,147 @@
       </c>
       <c r="C69" s="33" t="n">
         <f aca="false">C65-C66-C67-C68</f>
-        <v>265089.78</v>
+        <v>161192.7</v>
       </c>
       <c r="D69" s="33" t="n">
         <f aca="false">D65-D66-D67-D68</f>
-        <v>390676.063275</v>
+        <v>237557.741625</v>
       </c>
       <c r="E69" s="33" t="n">
         <f aca="false">E65-E66-E67-E68</f>
-        <v>575819.736060375</v>
+        <v>350137.745668125</v>
       </c>
       <c r="F69" s="33" t="n">
         <f aca="false">F65-F66-F67-F68</f>
-        <v>1257472.3004971</v>
+        <v>764629.082616234</v>
       </c>
       <c r="G69" s="33" t="n">
         <f aca="false">G65-G66-G67-G68</f>
-        <v>1699305.29447768</v>
+        <v>1033293.73369713</v>
       </c>
       <c r="H69" s="33" t="n">
         <f aca="false">H65-H66-H67-H68</f>
-        <v>2186539.6981865</v>
+        <v>1329565.54420116</v>
       </c>
       <c r="I69" s="33" t="n">
         <f aca="false">I65-I66-I67-I68</f>
-        <v>2716615.93531247</v>
+        <v>1651888.11683363</v>
       </c>
       <c r="J69" s="33" t="n">
         <f aca="false">J65-J66-J67-J68</f>
-        <v>1878341.70466248</v>
+        <v>1142160.10476582</v>
       </c>
       <c r="K69" s="33" t="n">
         <f aca="false">K65-K66-K67-K68</f>
-        <v>2337400.71562421</v>
+        <v>1421299.35123639</v>
       </c>
       <c r="L69" s="33" t="n">
         <f aca="false">L65-L66-L67-L68</f>
-        <v>2837575.2145304</v>
+        <v>1725439.62382569</v>
       </c>
       <c r="M69" s="33" t="n">
         <f aca="false">M65-M66-M67-M68</f>
-        <v>3069622.30702184</v>
+        <v>1866540.11199179</v>
       </c>
       <c r="N69" s="33" t="n">
         <f aca="false">N65-N66-N67-N68</f>
-        <v>3293547.75127607</v>
+        <v>2002702.08307208</v>
       </c>
       <c r="O69" s="33" t="n">
         <f aca="false">O65-O66-O67-O68</f>
-        <v>2966762.51198513</v>
+        <v>1803994.32813164</v>
       </c>
       <c r="P69" s="33" t="n">
         <f aca="false">P65-P66-P67-P68</f>
-        <v>2465302.10404924</v>
+        <v>1499072.13498528</v>
       </c>
       <c r="Q69" s="33" t="n">
         <f aca="false">Q65-Q66-Q67-Q68</f>
-        <v>2697124.26640751</v>
+        <v>1640035.85026079</v>
       </c>
       <c r="R69" s="33" t="n">
         <f aca="false">R65-R66-R67-R68</f>
-        <v>4868054.42180541</v>
+        <v>2960109.72583611</v>
       </c>
       <c r="S69" s="33" t="n">
         <f aca="false">S65-S66-S67-S68</f>
-        <v>5750637.28474645</v>
+        <v>3496780.41397503</v>
       </c>
       <c r="T69" s="33" t="n">
         <f aca="false">T65-T66-T67-T68</f>
-        <v>6690068.1772149</v>
+        <v>4068018.58853007</v>
       </c>
       <c r="U69" s="33" t="n">
         <f aca="false">U65-U66-U67-U68</f>
-        <v>7683142.20159674</v>
+        <v>4671875.45275915</v>
       </c>
       <c r="V69" s="33" t="n">
         <f aca="false">V65-V66-V67-V68</f>
-        <v>4986748.0938713</v>
+        <v>3032283.58886928</v>
       </c>
       <c r="W69" s="33" t="n">
         <f aca="false">W65-W66-W67-W68</f>
-        <v>5890900.00340903</v>
+        <v>3582069.73116621</v>
       </c>
       <c r="X69" s="33" t="n">
         <f aca="false">X65-X66-X67-X68</f>
-        <v>6846533.45254412</v>
+        <v>4163160.16730599</v>
       </c>
       <c r="Y69" s="33" t="n">
         <f aca="false">Y65-Y66-Y67-Y68</f>
-        <v>7137084.34170508</v>
+        <v>4339834.96145028</v>
       </c>
       <c r="Z69" s="33" t="n">
         <f aca="false">Z65-Z66-Z67-Z68</f>
-        <v>7417465.9497454</v>
+        <v>4510326.13779952</v>
       </c>
       <c r="AA69" s="33" t="n">
         <f aca="false">AA65-AA66-AA67-AA68</f>
-        <v>6309481.22920345</v>
+        <v>3836595.71838123</v>
       </c>
       <c r="AB69" s="33" t="n">
         <f aca="false">AB65-AB66-AB67-AB68</f>
-        <v>5003885.176636</v>
+        <v>3042704.10617842</v>
       </c>
       <c r="AC69" s="33" t="n">
         <f aca="false">AC65-AC66-AC67-AC68</f>
-        <v>5266147.33245374</v>
+        <v>3202177.41746217</v>
       </c>
       <c r="AD69" s="33" t="n">
         <f aca="false">AD65-AD66-AD67-AD68</f>
-        <v>9198717.18802976</v>
+        <v>5593448.60475166</v>
       </c>
       <c r="AE69" s="33" t="n">
         <f aca="false">AE65-AE66-AE67-AE68</f>
-        <v>10566334.8795936</v>
+        <v>6425053.61144389</v>
       </c>
       <c r="AF69" s="33" t="n">
         <f aca="false">AF65-AF66-AF67-AF68</f>
-        <v>11998265.1745176</v>
+        <v>7295765.07550184</v>
       </c>
       <c r="AG69" s="33" t="n">
         <f aca="false">AG65-AG66-AG67-AG68</f>
-        <v>13490882.348027</v>
+        <v>8203378.30851421</v>
       </c>
       <c r="AH69" s="33" t="n">
         <f aca="false">AH65-AH66-AH67-AH68</f>
-        <v>8594706.11036678</v>
+        <v>5226168.59705613</v>
       </c>
       <c r="AI69" s="33" t="n">
         <f aca="false">AI65-AI66-AI67-AI68</f>
-        <v>9986725.02656693</v>
+        <v>6072611.21567906</v>
       </c>
       <c r="AJ69" s="33" t="n">
         <f aca="false">AJ65-AJ66-AJ67-AJ68</f>
-        <v>11436985.3957079</v>
+        <v>6954468.617367</v>
       </c>
       <c r="AK69" s="33" t="n">
         <f aca="false">AK65-AK66-AK67-AK68</f>
-        <v>11765687.8018581</v>
+        <v>7154342.14075915</v>
       </c>
       <c r="AL69" s="33" t="n">
         <f aca="false">AL65-AL66-AL67-AL68</f>
-        <v>12082885.6237931</v>
+        <v>7347220.09083258</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14607,147 +14607,147 @@
       </c>
       <c r="C75" s="33" t="n">
         <f aca="false">C69-C74</f>
-        <v>-1134910.22</v>
+        <v>-1238807.3</v>
       </c>
       <c r="D75" s="33" t="n">
         <f aca="false">D69-D74</f>
-        <v>-209323.936725</v>
+        <v>-362442.258375</v>
       </c>
       <c r="E75" s="33" t="n">
         <f aca="false">E69-E74</f>
-        <v>-24180.263939625</v>
+        <v>-249862.254331875</v>
       </c>
       <c r="F75" s="33" t="n">
         <f aca="false">F69-F74</f>
-        <v>657472.300497103</v>
+        <v>164629.082616234</v>
       </c>
       <c r="G75" s="33" t="n">
         <f aca="false">G69-G74</f>
-        <v>1099305.29447768</v>
+        <v>433293.733697133</v>
       </c>
       <c r="H75" s="33" t="n">
         <f aca="false">H69-H74</f>
-        <v>1586539.6981865</v>
+        <v>729565.544201164</v>
       </c>
       <c r="I75" s="33" t="n">
         <f aca="false">I69-I74</f>
-        <v>2116615.93531247</v>
+        <v>1051888.11683363</v>
       </c>
       <c r="J75" s="33" t="n">
         <f aca="false">J69-J74</f>
-        <v>1278341.70466248</v>
+        <v>542160.104765819</v>
       </c>
       <c r="K75" s="33" t="n">
         <f aca="false">K69-K74</f>
-        <v>1737400.71562421</v>
+        <v>821299.351236392</v>
       </c>
       <c r="L75" s="33" t="n">
         <f aca="false">L69-L74</f>
-        <v>2237575.2145304</v>
+        <v>1125439.62382569</v>
       </c>
       <c r="M75" s="33" t="n">
         <f aca="false">M69-M74</f>
-        <v>2469622.30702184</v>
+        <v>1266540.11199179</v>
       </c>
       <c r="N75" s="33" t="n">
         <f aca="false">N69-N74</f>
-        <v>2693547.75127607</v>
+        <v>1402702.08307208</v>
       </c>
       <c r="O75" s="33" t="n">
         <f aca="false">O69-O74</f>
-        <v>1706762.51198513</v>
+        <v>543994.328131642</v>
       </c>
       <c r="P75" s="33" t="n">
         <f aca="false">P69-P74</f>
-        <v>1205302.10404924</v>
+        <v>239072.134985277</v>
       </c>
       <c r="Q75" s="33" t="n">
         <f aca="false">Q69-Q74</f>
-        <v>1437124.26640751</v>
+        <v>380035.850260792</v>
       </c>
       <c r="R75" s="33" t="n">
         <f aca="false">R69-R74</f>
-        <v>3608054.42180541</v>
+        <v>1700109.72583611</v>
       </c>
       <c r="S75" s="33" t="n">
         <f aca="false">S69-S74</f>
-        <v>4490637.28474645</v>
+        <v>2236780.41397503</v>
       </c>
       <c r="T75" s="33" t="n">
         <f aca="false">T69-T74</f>
-        <v>5430068.1772149</v>
+        <v>2808018.58853007</v>
       </c>
       <c r="U75" s="33" t="n">
         <f aca="false">U69-U74</f>
-        <v>6423142.20159674</v>
+        <v>3411875.45275915</v>
       </c>
       <c r="V75" s="33" t="n">
         <f aca="false">V69-V74</f>
-        <v>3726748.0938713</v>
+        <v>1772283.58886928</v>
       </c>
       <c r="W75" s="33" t="n">
         <f aca="false">W69-W74</f>
-        <v>4630900.00340903</v>
+        <v>2322069.73116621</v>
       </c>
       <c r="X75" s="33" t="n">
         <f aca="false">X69-X74</f>
-        <v>5586533.45254412</v>
+        <v>2903160.16730599</v>
       </c>
       <c r="Y75" s="33" t="n">
         <f aca="false">Y69-Y74</f>
-        <v>5877084.34170508</v>
+        <v>3079834.96145028</v>
       </c>
       <c r="Z75" s="33" t="n">
         <f aca="false">Z69-Z74</f>
-        <v>6157465.9497454</v>
+        <v>3250326.13779952</v>
       </c>
       <c r="AA75" s="33" t="n">
         <f aca="false">AA69-AA74</f>
-        <v>4469481.22920345</v>
+        <v>1996595.71838123</v>
       </c>
       <c r="AB75" s="33" t="n">
         <f aca="false">AB69-AB74</f>
-        <v>3163885.17663599</v>
+        <v>1202704.10617842</v>
       </c>
       <c r="AC75" s="33" t="n">
         <f aca="false">AC69-AC74</f>
-        <v>3426147.33245374</v>
+        <v>1362177.41746217</v>
       </c>
       <c r="AD75" s="33" t="n">
         <f aca="false">AD69-AD74</f>
-        <v>7358717.18802976</v>
+        <v>3753448.60475166</v>
       </c>
       <c r="AE75" s="33" t="n">
         <f aca="false">AE69-AE74</f>
-        <v>8726334.87959359</v>
+        <v>4585053.61144389</v>
       </c>
       <c r="AF75" s="33" t="n">
         <f aca="false">AF69-AF74</f>
-        <v>10158265.1745176</v>
+        <v>5455765.07550184</v>
       </c>
       <c r="AG75" s="33" t="n">
         <f aca="false">AG69-AG74</f>
-        <v>11650882.348027</v>
+        <v>6363378.30851421</v>
       </c>
       <c r="AH75" s="33" t="n">
         <f aca="false">AH69-AH74</f>
-        <v>6754706.11036678</v>
+        <v>3386168.59705613</v>
       </c>
       <c r="AI75" s="33" t="n">
         <f aca="false">AI69-AI74</f>
-        <v>8146725.02656693</v>
+        <v>4232611.21567906</v>
       </c>
       <c r="AJ75" s="33" t="n">
         <f aca="false">AJ69-AJ74</f>
-        <v>9596985.39570788</v>
+        <v>5114468.617367</v>
       </c>
       <c r="AK75" s="33" t="n">
         <f aca="false">AK69-AK74</f>
-        <v>9925687.80185811</v>
+        <v>5314342.14075915</v>
       </c>
       <c r="AL75" s="33" t="n">
         <f aca="false">AL69-AL74</f>
-        <v>10242885.6237931</v>
+        <v>5507220.09083258</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14759,147 +14759,147 @@
       </c>
       <c r="C76" s="33" t="n">
         <f aca="false">C75</f>
-        <v>-1134910.22</v>
+        <v>-1238807.3</v>
       </c>
       <c r="D76" s="33" t="n">
         <f aca="false">C76+D75</f>
-        <v>-1344234.156725</v>
+        <v>-1601249.558375</v>
       </c>
       <c r="E76" s="33" t="n">
         <f aca="false">D76+E75</f>
-        <v>-1368414.42066462</v>
+        <v>-1851111.81270688</v>
       </c>
       <c r="F76" s="33" t="n">
         <f aca="false">E76+F75</f>
-        <v>-710942.120167522</v>
+        <v>-1686482.73009064</v>
       </c>
       <c r="G76" s="33" t="n">
         <f aca="false">F76+G75</f>
-        <v>388363.174310154</v>
+        <v>-1253188.99639351</v>
       </c>
       <c r="H76" s="33" t="n">
         <f aca="false">G76+H75</f>
-        <v>1974902.87249665</v>
+        <v>-523623.452192344</v>
       </c>
       <c r="I76" s="33" t="n">
         <f aca="false">H76+I75</f>
-        <v>4091518.80780912</v>
+        <v>528264.66464129</v>
       </c>
       <c r="J76" s="33" t="n">
         <f aca="false">I76+J75</f>
-        <v>5369860.5124716</v>
+        <v>1070424.76940711</v>
       </c>
       <c r="K76" s="33" t="n">
         <f aca="false">J76+K75</f>
-        <v>7107261.22809581</v>
+        <v>1891724.1206435</v>
       </c>
       <c r="L76" s="33" t="n">
         <f aca="false">K76+L75</f>
-        <v>9344836.44262621</v>
+        <v>3017163.74446919</v>
       </c>
       <c r="M76" s="33" t="n">
         <f aca="false">L76+M75</f>
-        <v>11814458.749648</v>
+        <v>4283703.85646098</v>
       </c>
       <c r="N76" s="33" t="n">
         <f aca="false">M76+N75</f>
-        <v>14508006.5009241</v>
+        <v>5686405.93953305</v>
       </c>
       <c r="O76" s="33" t="n">
         <f aca="false">N76+O75</f>
-        <v>16214769.0129092</v>
+        <v>6230400.2676647</v>
       </c>
       <c r="P76" s="33" t="n">
         <f aca="false">O76+P75</f>
-        <v>17420071.1169585</v>
+        <v>6469472.40264997</v>
       </c>
       <c r="Q76" s="33" t="n">
         <f aca="false">P76+Q75</f>
-        <v>18857195.383366</v>
+        <v>6849508.25291076</v>
       </c>
       <c r="R76" s="33" t="n">
         <f aca="false">Q76+R75</f>
-        <v>22465249.8051714</v>
+        <v>8549617.97874687</v>
       </c>
       <c r="S76" s="33" t="n">
         <f aca="false">R76+S75</f>
-        <v>26955887.0899179</v>
+        <v>10786398.3927219</v>
       </c>
       <c r="T76" s="33" t="n">
         <f aca="false">S76+T75</f>
-        <v>32385955.2671328</v>
+        <v>13594416.981252</v>
       </c>
       <c r="U76" s="33" t="n">
         <f aca="false">T76+U75</f>
-        <v>38809097.4687295</v>
+        <v>17006292.4340111</v>
       </c>
       <c r="V76" s="33" t="n">
         <f aca="false">U76+V75</f>
-        <v>42535845.5626008</v>
+        <v>18778576.0228804</v>
       </c>
       <c r="W76" s="33" t="n">
         <f aca="false">V76+W75</f>
-        <v>47166745.5660098</v>
+        <v>21100645.7540466</v>
       </c>
       <c r="X76" s="33" t="n">
         <f aca="false">W76+X75</f>
-        <v>52753279.0185539</v>
+        <v>24003805.9213526</v>
       </c>
       <c r="Y76" s="33" t="n">
         <f aca="false">X76+Y75</f>
-        <v>58630363.360259</v>
+        <v>27083640.8828029</v>
       </c>
       <c r="Z76" s="33" t="n">
         <f aca="false">Y76+Z75</f>
-        <v>64787829.3100044</v>
+        <v>30333967.0206024</v>
       </c>
       <c r="AA76" s="33" t="n">
         <f aca="false">Z76+AA75</f>
-        <v>69257310.5392079</v>
+        <v>32330562.7389836</v>
       </c>
       <c r="AB76" s="33" t="n">
         <f aca="false">AA76+AB75</f>
-        <v>72421195.7158439</v>
+        <v>33533266.8451621</v>
       </c>
       <c r="AC76" s="33" t="n">
         <f aca="false">AB76+AC75</f>
-        <v>75847343.0482976</v>
+        <v>34895444.2626242</v>
       </c>
       <c r="AD76" s="33" t="n">
         <f aca="false">AC76+AD75</f>
-        <v>83206060.2363274</v>
+        <v>38648892.8673759</v>
       </c>
       <c r="AE76" s="33" t="n">
         <f aca="false">AD76+AE75</f>
-        <v>91932395.115921</v>
+        <v>43233946.4788198</v>
       </c>
       <c r="AF76" s="33" t="n">
         <f aca="false">AE76+AF75</f>
-        <v>102090660.290439</v>
+        <v>48689711.5543216</v>
       </c>
       <c r="AG76" s="33" t="n">
         <f aca="false">AF76+AG75</f>
-        <v>113741542.638466</v>
+        <v>55053089.8628358</v>
       </c>
       <c r="AH76" s="33" t="n">
         <f aca="false">AG76+AH75</f>
-        <v>120496248.748832</v>
+        <v>58439258.459892</v>
       </c>
       <c r="AI76" s="33" t="n">
         <f aca="false">AH76+AI75</f>
-        <v>128642973.775399</v>
+        <v>62671869.675571</v>
       </c>
       <c r="AJ76" s="33" t="n">
         <f aca="false">AI76+AJ75</f>
-        <v>138239959.171107</v>
+        <v>67786338.292938</v>
       </c>
       <c r="AK76" s="33" t="n">
         <f aca="false">AJ76+AK75</f>
-        <v>148165646.972965</v>
+        <v>73100680.4336972</v>
       </c>
       <c r="AL76" s="33" t="n">
         <f aca="false">AK76+AL75</f>
-        <v>158408532.596758</v>
+        <v>78607900.5245298</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15073,13 +15073,13 @@
         <f aca="false">IF(F76&gt;=0,F$4,"")</f>
         <v/>
       </c>
-      <c r="G78" s="34" t="n">
+      <c r="G78" s="34" t="str">
         <f aca="false">IF(G76&gt;=0,G$4,"")</f>
-        <v>5</v>
-      </c>
-      <c r="H78" s="34" t="n">
+        <v/>
+      </c>
+      <c r="H78" s="34" t="str">
         <f aca="false">IF(H76&gt;=0,H$4,"")</f>
-        <v>6</v>
+        <v/>
       </c>
       <c r="I78" s="34" t="n">
         <f aca="false">IF(I76&gt;=0,I$4,"")</f>
@@ -15422,11 +15422,11 @@
       </c>
       <c r="C16" s="35" t="n">
         <f aca="false">C13*Допущения!$C$6*(1-Допущения!$C$13)</f>
-        <v>47858955.7554621</v>
+        <v>34184968.3967586</v>
       </c>
       <c r="D16" s="35" t="n">
         <f aca="false">IF($C$11=0,0,C16/$C$11)</f>
-        <v>46154.5877879895</v>
+        <v>32967.5627057068</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>172</v>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="C21" s="36" t="n">
         <f aca="false">IF(Допущения!$D$22*Допущения!$C$6*(1-Допущения!$C$13)=0,0,C5/(Допущения!$D$22*Допущения!$C$6*(1-Допущения!$C$13)))</f>
-        <v>61.3647520864016</v>
+        <v>85.9106529209622</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -15688,7 +15688,7 @@
       </c>
       <c r="H5" s="35" t="n">
         <f aca="false">G5*Допущения!$C$6</f>
-        <v>168000000</v>
+        <v>120000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15714,7 +15714,7 @@
       </c>
       <c r="H6" s="35" t="n">
         <f aca="false">G6*Допущения!$C$6</f>
-        <v>705600000</v>
+        <v>504000000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15740,7 +15740,7 @@
       </c>
       <c r="H7" s="35" t="n">
         <f aca="false">G7*Допущения!$C$6</f>
-        <v>201600000</v>
+        <v>144000000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15766,7 +15766,7 @@
       </c>
       <c r="H8" s="35" t="n">
         <f aca="false">G8*Допущения!$C$6</f>
-        <v>189000000</v>
+        <v>135000000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15792,7 +15792,7 @@
       </c>
       <c r="H9" s="35" t="n">
         <f aca="false">G9*Допущения!$C$6</f>
-        <v>84000000</v>
+        <v>60000000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15818,7 +15818,7 @@
       </c>
       <c r="H10" s="35" t="n">
         <f aca="false">G10*Допущения!$C$6</f>
-        <v>120960000</v>
+        <v>86400000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="H11" s="13" t="n">
         <f aca="false">SUM(H5:H10)</f>
-        <v>1469160000</v>
+        <v>1049400000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs(business): scenario table and the fee-vs-subscription argument
New organizers per year were transposed across scenarios and founder pay
was listed per scenario instead of per year. The average base-case
organizer sells about 112 paid tickets a month, above the 86 break-even,
so the fee wins even per paying organizer. xlsx rebuilt, three text
cells change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G6Artzpr7bcnkUftwxLCYd
</commit_message>
<xml_diff>
--- a/docs/business/finmodel.xlsx
+++ b/docs/business/finmodel.xlsx
@@ -139,7 +139,7 @@
     <t xml:space="preserve">Маржа, % от цены билета</t>
   </si>
   <si>
-    <t xml:space="preserve">в spec.md было ~2% при сборе 5% и эквайринге 2,5%</t>
+    <t xml:space="preserve">в первой версии spec.md было ~2% при сборе 5% и эквайринге 2,5%</t>
   </si>
   <si>
     <t xml:space="preserve">На одного организатора</t>
@@ -562,7 +562,7 @@
     <t xml:space="preserve">Платных билетов в месяц у организатора, при которых сбор = подписке</t>
   </si>
   <si>
-    <t xml:space="preserve">меньше — организатору выгоднее процент (типичный МСБ), больше — подписка</t>
+    <t xml:space="preserve">меньше — организатору выгоднее процент, больше — подписка; средний организатор базового сценария (строка 22) выше точки равенства</t>
   </si>
   <si>
     <t xml:space="preserve">Платных билетов в месяц у организатора в базовом сценарии</t>
@@ -571,7 +571,7 @@
     <t xml:space="preserve">Вывод</t>
   </si>
   <si>
-    <t xml:space="preserve">Сервисный сбор платит покупатель, поэтому организатору вход бесплатный — это главный аргумент для МСБ против крупных площадок, где обычно платят обе стороны (схема «10/10» у Ticketscloud: сбор с покупателя и комиссия с организатора). Подписка выгоднее только крупным организаторам с объёмом выше точки равенства, но их на старте нет, а у мелких она отсекает половину клиентов.</t>
+    <t xml:space="preserve">Сервисный сбор платит покупатель, поэтому организатору вход бесплатный — это главный аргумент для МСБ против крупных площадок, где обычно платят обе стороны (схема «10/10» у Ticketscloud: сбор с покупателя и комиссия с организатора). Подписка выгоднее организаторам с объёмом выше точки равенства, а средний организатор базового сценария — около 112 платных билетов в месяц — как раз выше неё. Поэтому сбор приносит больше подписки даже с каждого платящего организатора (примерно в 1,3 раза), а то, что подписку платит только половина организаторов, удваивает разрыв.</t>
   </si>
   <si>
     <t xml:space="preserve">Рынок снизу вверх: МСБ-организаторы Казахстана</t>
@@ -2286,11 +2286,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="47611281"/>
-        <c:axId val="67006473"/>
+        <c:axId val="78995315"/>
+        <c:axId val="53708243"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="47611281"/>
+        <c:axId val="78995315"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2356,7 +2356,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67006473"/>
+        <c:crossAx val="53708243"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2364,7 +2364,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67006473"/>
+        <c:axId val="53708243"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2440,7 +2440,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47611281"/>
+        <c:crossAx val="78995315"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>